<commit_message>
Added additional placeholder values for required columns that are missing data in the source
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\serverfiles\projects\python\mohccn-omop-etl\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DC2F136-2D4F-4C09-9EE6-29BDA8F88293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989FB45E-C548-4CD8-A12E-2343B8EFF2CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5959937F-EF1A-4EF7-9756-DEAA4796FC13}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4577" uniqueCount="730">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4579" uniqueCount="730">
   <si>
     <t>mCODE Profile Name</t>
   </si>
@@ -13163,6 +13163,9 @@
       <c r="J506" s="3" t="s">
         <v>308</v>
       </c>
+      <c r="K506" s="3" t="s">
+        <v>698</v>
+      </c>
     </row>
     <row r="507" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E507" s="3" t="s">
@@ -13190,6 +13193,9 @@
       </c>
       <c r="H508" s="7" t="s">
         <v>228</v>
+      </c>
+      <c r="K508" s="3" t="s">
+        <v>697</v>
       </c>
     </row>
     <row r="509" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Added placeholder values for comorbidity concept id and start date if missing in source data.  Changed missing dob interval message to not display on the screen
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\serverfiles\projects\dhdp\mohccn-omop-etl\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\serverfiles\projects\python\mohccn-omop-etl\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13B69D8E-A767-402C-96BF-08E1761BA9B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E6A1A96-F0D5-4BC8-8D15-1ACE1BB15999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5959937F-EF1A-4EF7-9756-DEAA4796FC13}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3075" uniqueCount="615">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3077" uniqueCount="615">
   <si>
     <t>Sample Registration</t>
   </si>
@@ -12813,6 +12813,9 @@
       <c r="J506" s="2" t="s">
         <v>193</v>
       </c>
+      <c r="K506" s="2" t="s">
+        <v>584</v>
+      </c>
     </row>
     <row r="507" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E507" s="2" t="s">
@@ -12840,6 +12843,9 @@
       </c>
       <c r="H508" s="6" t="s">
         <v>113</v>
+      </c>
+      <c r="K508" s="2" t="s">
+        <v>583</v>
       </c>
     </row>
     <row r="509" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated tranformation model for exposure.tobacco_type and surgery.margin_types_*.
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\serverfiles\projects\dhdp\mohccn-omop-etl\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD64129-D1F8-4DAE-921D-C11AC951EB19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E729826-CDB9-41C9-9474-8DF622B9B916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5959937F-EF1A-4EF7-9756-DEAA4796FC13}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5959937F-EF1A-4EF7-9756-DEAA4796FC13}"/>
   </bookViews>
   <sheets>
     <sheet name="Transformation Model" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3384" uniqueCount="621">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3380" uniqueCount="624">
   <si>
     <t>Sample Registration</t>
   </si>
@@ -1690,9 +1690,6 @@
     <t>2000-01-01</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>Concatenate Values</t>
   </si>
   <si>
@@ -1904,6 +1901,18 @@
   </si>
   <si>
     <t>treatment_type</t>
+  </si>
+  <si>
+    <t>$.donors[].exposures[].tobacco_type[]</t>
+  </si>
+  <si>
+    <t>$.donors[].primary_diagnoses[].treatments[].surgeries[].margin_types_involved[]</t>
+  </si>
+  <si>
+    <t>$.donors[].primary_diagnoses[].treatments[].surgeries[].margin_types_not_involved[]</t>
+  </si>
+  <si>
+    <t>$.donors[].primary_diagnoses[].treatments[].surgeries[].margin_types_not_assessed[]</t>
   </si>
 </sst>
 </file>
@@ -2383,7 +2392,7 @@
         <v>127</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="L1" s="5" t="s">
         <v>128</v>
@@ -2438,7 +2447,7 @@
         <v>133</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -2497,10 +2506,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D6" s="2" t="s">
+        <v>573</v>
+      </c>
+      <c r="E6" s="2" t="s">
         <v>574</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>575</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>132</v>
@@ -2564,7 +2573,7 @@
         <v>133</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -2641,7 +2650,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
@@ -2665,7 +2674,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
@@ -2689,7 +2698,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
@@ -2713,7 +2722,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
@@ -2737,7 +2746,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
@@ -2761,12 +2770,12 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="D17" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>147</v>
@@ -2785,7 +2794,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -2809,7 +2818,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
@@ -2833,7 +2842,7 @@
         <v>OMOP Patient Person</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
@@ -2844,7 +2853,7 @@
         <v>149</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>19</v>
@@ -2865,7 +2874,7 @@
         <v>149</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>34</v>
@@ -2886,7 +2895,7 @@
         <v>149</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G22" s="2" t="s">
         <v>50</v>
@@ -2907,7 +2916,7 @@
         <v>149</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="G23" s="2" t="s">
         <v>90</v>
@@ -2928,7 +2937,7 @@
         <v>150</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>19</v>
@@ -2954,7 +2963,7 @@
         <v>150</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>34</v>
@@ -2980,7 +2989,7 @@
         <v>150</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G26" s="2" t="s">
         <v>50</v>
@@ -3006,7 +3015,7 @@
         <v>150</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>90</v>
@@ -3015,13 +3024,13 @@
         <v>91</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
@@ -3038,7 +3047,7 @@
         <v>133</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="G28" s="2" t="s">
         <v>133</v>
@@ -3093,7 +3102,7 @@
         <v>543</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>132</v>
@@ -3105,7 +3114,7 @@
         <v>133</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
@@ -3113,7 +3122,7 @@
         <v>543</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>132</v>
@@ -3133,25 +3142,25 @@
         <v>543</v>
       </c>
       <c r="E33" s="2" t="s">
+        <v>559</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="I33" s="14" t="s">
         <v>560</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="I33" s="14" t="s">
-        <v>561</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="3" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>543</v>
@@ -3160,7 +3169,7 @@
         <v>133</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>9</v>
@@ -3177,7 +3186,7 @@
         <v>133</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>9</v>
@@ -3194,7 +3203,7 @@
         <v>133</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G36" s="2" t="s">
         <v>9</v>
@@ -3211,7 +3220,7 @@
         <v>133</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G37" s="2" t="s">
         <v>9</v>
@@ -3223,10 +3232,10 @@
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B38" s="2"/>
       <c r="D38" s="2" t="s">
+        <v>593</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>594</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>595</v>
       </c>
       <c r="F38" s="2" t="s">
         <v>154</v>
@@ -3238,10 +3247,10 @@
         <v>133</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
@@ -3265,7 +3274,7 @@
         <v>2</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
@@ -3282,10 +3291,10 @@
         <v>133</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
@@ -3308,7 +3317,7 @@
         <v>159</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>160</v>
@@ -3348,7 +3357,7 @@
         <v>12</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
@@ -3368,7 +3377,7 @@
         <v>12</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
@@ -3388,12 +3397,12 @@
         <v>12</v>
       </c>
       <c r="K45" s="2" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E46" s="2" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>154</v>
@@ -3405,12 +3414,12 @@
         <v>133</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E47" s="2" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="F47" s="2" t="s">
         <v>154</v>
@@ -3422,7 +3431,7 @@
         <v>133</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="48" spans="1:12" ht="27" x14ac:dyDescent="0.25">
@@ -3445,7 +3454,7 @@
         <v>2</v>
       </c>
       <c r="K48" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
@@ -3488,7 +3497,7 @@
         <v>10</v>
       </c>
       <c r="K50" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
@@ -3555,7 +3564,7 @@
         <v>13</v>
       </c>
       <c r="K53" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
@@ -3642,7 +3651,7 @@
         <v>133</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>34</v>
@@ -3651,7 +3660,7 @@
         <v>20</v>
       </c>
       <c r="K59" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
@@ -3672,7 +3681,7 @@
         <v>20</v>
       </c>
       <c r="K60" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
@@ -3695,7 +3704,7 @@
         <v>193</v>
       </c>
       <c r="K61" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
@@ -3733,7 +3742,7 @@
       </c>
       <c r="I63" s="2"/>
       <c r="K63" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
@@ -3780,7 +3789,7 @@
         <v>20</v>
       </c>
       <c r="K65" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="66" spans="2:12" x14ac:dyDescent="0.25">
@@ -3841,7 +3850,7 @@
         <v>193</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="69" spans="2:12" x14ac:dyDescent="0.25">
@@ -3919,7 +3928,7 @@
         <v>OMOP Primary Dx Episode</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="73" spans="2:12" x14ac:dyDescent="0.25">
@@ -3940,7 +3949,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K73" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="74" spans="2:12" x14ac:dyDescent="0.25">
@@ -3986,7 +3995,7 @@
         <v>20</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="76" spans="2:12" x14ac:dyDescent="0.25">
@@ -4047,7 +4056,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K78" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="79" spans="2:12" x14ac:dyDescent="0.25">
@@ -4127,7 +4136,7 @@
         <v>20</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="83" spans="2:12" x14ac:dyDescent="0.25">
@@ -4188,7 +4197,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K85" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.25">
@@ -4231,7 +4240,7 @@
         <v>39</v>
       </c>
       <c r="K87" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="88" spans="2:12" x14ac:dyDescent="0.25">
@@ -4271,7 +4280,7 @@
         <v>20</v>
       </c>
       <c r="K89" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="90" spans="2:12" x14ac:dyDescent="0.25">
@@ -4331,7 +4340,7 @@
         <v>37</v>
       </c>
       <c r="K92" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="93" spans="2:12" x14ac:dyDescent="0.25">
@@ -4369,7 +4378,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K94" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="95" spans="2:12" x14ac:dyDescent="0.25">
@@ -4415,7 +4424,7 @@
         <v>20</v>
       </c>
       <c r="K96" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="97" spans="2:12" x14ac:dyDescent="0.25">
@@ -4476,7 +4485,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="100" spans="2:12" x14ac:dyDescent="0.25">
@@ -4519,7 +4528,7 @@
         <v>44</v>
       </c>
       <c r="K101" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="102" spans="2:12" x14ac:dyDescent="0.25">
@@ -4559,7 +4568,7 @@
         <v>20</v>
       </c>
       <c r="K103" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="104" spans="2:12" x14ac:dyDescent="0.25">
@@ -4620,7 +4629,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K106" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="107" spans="2:12" x14ac:dyDescent="0.25">
@@ -4663,7 +4672,7 @@
         <v>45</v>
       </c>
       <c r="K108" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="109" spans="2:12" x14ac:dyDescent="0.25">
@@ -4703,7 +4712,7 @@
         <v>20</v>
       </c>
       <c r="K110" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="111" spans="2:12" x14ac:dyDescent="0.25">
@@ -4764,7 +4773,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K113" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="114" spans="2:12" x14ac:dyDescent="0.25">
@@ -4807,7 +4816,7 @@
         <v>46</v>
       </c>
       <c r="K115" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="116" spans="2:12" x14ac:dyDescent="0.25">
@@ -4847,7 +4856,7 @@
         <v>20</v>
       </c>
       <c r="K117" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="118" spans="2:12" x14ac:dyDescent="0.25">
@@ -4867,7 +4876,7 @@
         <v>40</v>
       </c>
       <c r="K118" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="119" spans="2:12" x14ac:dyDescent="0.25">
@@ -4999,7 +5008,7 @@
         <v>20</v>
       </c>
       <c r="K125" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="126" spans="2:12" x14ac:dyDescent="0.25">
@@ -5060,7 +5069,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K128" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="129" spans="2:12" x14ac:dyDescent="0.25">
@@ -5103,7 +5112,7 @@
         <v>47</v>
       </c>
       <c r="K130" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="131" spans="2:12" x14ac:dyDescent="0.25">
@@ -5143,7 +5152,7 @@
         <v>20</v>
       </c>
       <c r="K132" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="133" spans="2:12" x14ac:dyDescent="0.25">
@@ -5204,7 +5213,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K135" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="136" spans="2:12" x14ac:dyDescent="0.25">
@@ -5247,7 +5256,7 @@
         <v>48</v>
       </c>
       <c r="K137" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="138" spans="2:12" x14ac:dyDescent="0.25">
@@ -5287,7 +5296,7 @@
         <v>20</v>
       </c>
       <c r="K139" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="140" spans="2:12" x14ac:dyDescent="0.25">
@@ -5348,7 +5357,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K142" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="143" spans="2:12" x14ac:dyDescent="0.25">
@@ -5391,7 +5400,7 @@
         <v>49</v>
       </c>
       <c r="K144" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.25">
@@ -5431,7 +5440,7 @@
         <v>20</v>
       </c>
       <c r="K146" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.25">
@@ -5451,7 +5460,7 @@
         <v>42</v>
       </c>
       <c r="K147" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="148" spans="1:12" x14ac:dyDescent="0.25">
@@ -5506,7 +5515,7 @@
         <v>OMOP Primary Dx Condition</v>
       </c>
       <c r="K150" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.25">
@@ -5580,7 +5589,7 @@
         <v>133</v>
       </c>
       <c r="F154" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G154" s="2" t="s">
         <v>50</v>
@@ -5589,7 +5598,7 @@
         <v>21</v>
       </c>
       <c r="K154" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
@@ -5600,7 +5609,7 @@
         <v>133</v>
       </c>
       <c r="F155" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G155" s="2" t="s">
         <v>50</v>
@@ -5609,7 +5618,7 @@
         <v>52</v>
       </c>
       <c r="K155" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
@@ -5620,7 +5629,7 @@
         <v>133</v>
       </c>
       <c r="F156" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G156" s="2" t="s">
         <v>50</v>
@@ -5648,7 +5657,7 @@
         <v>21</v>
       </c>
       <c r="K157" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
@@ -5725,7 +5734,7 @@
         <v>52</v>
       </c>
       <c r="K161" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="162" spans="2:12" x14ac:dyDescent="0.25">
@@ -5782,7 +5791,7 @@
         <v>21</v>
       </c>
       <c r="K164" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="165" spans="2:12" x14ac:dyDescent="0.25">
@@ -5799,13 +5808,13 @@
         <v>133</v>
       </c>
       <c r="I165" s="3" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="J165" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L165" s="2" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="166" spans="2:12" x14ac:dyDescent="0.25">
@@ -5822,7 +5831,7 @@
         <v>52</v>
       </c>
       <c r="K166" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="167" spans="2:12" x14ac:dyDescent="0.25">
@@ -5843,7 +5852,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K167" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="168" spans="2:12" x14ac:dyDescent="0.25">
@@ -5886,7 +5895,7 @@
         <v>54</v>
       </c>
       <c r="K169" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="170" spans="2:12" x14ac:dyDescent="0.25">
@@ -5926,7 +5935,7 @@
         <v>21</v>
       </c>
       <c r="K171" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="172" spans="2:12" x14ac:dyDescent="0.25">
@@ -5969,7 +5978,7 @@
         <v>530</v>
       </c>
       <c r="K173" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="174" spans="2:12" x14ac:dyDescent="0.25">
@@ -6003,7 +6012,7 @@
         <v>52</v>
       </c>
       <c r="K175" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="176" spans="2:12" x14ac:dyDescent="0.25">
@@ -6024,7 +6033,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K176" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
@@ -6086,10 +6095,10 @@
     </row>
     <row r="180" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A180" s="5" t="s">
+        <v>607</v>
+      </c>
+      <c r="B180" s="3" t="s">
         <v>608</v>
-      </c>
-      <c r="B180" s="3" t="s">
-        <v>609</v>
       </c>
       <c r="D180" s="2" t="s">
         <v>143</v>
@@ -6098,7 +6107,7 @@
         <v>255</v>
       </c>
       <c r="F180" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G180" s="2" t="s">
         <v>50</v>
@@ -6107,7 +6116,7 @@
         <v>21</v>
       </c>
       <c r="K180" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
@@ -6115,13 +6124,13 @@
         <v>256</v>
       </c>
       <c r="F181" s="2" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="G181" s="2" t="s">
         <v>50</v>
       </c>
       <c r="H181" s="6" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
@@ -6132,7 +6141,7 @@
         <v>258</v>
       </c>
       <c r="F182" s="2" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="G182" s="2" t="s">
         <v>133</v>
@@ -6155,10 +6164,10 @@
         <v>133</v>
       </c>
       <c r="I183" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K183" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
@@ -6178,7 +6187,7 @@
         <v>56</v>
       </c>
       <c r="I184" s="3" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
@@ -6198,12 +6207,12 @@
         <v>133</v>
       </c>
       <c r="I185" s="3" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="186" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B186" s="3" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D186" s="2" t="s">
         <v>210</v>
@@ -6225,7 +6234,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K186" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
@@ -6233,7 +6242,7 @@
         <v>211</v>
       </c>
       <c r="F187" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G187" s="2" t="s">
         <v>50</v>
@@ -6246,7 +6255,7 @@
         <v>OMOP Treatment Episode Procedure Occurrence</v>
       </c>
       <c r="K187" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="188" spans="1:12" x14ac:dyDescent="0.25">
@@ -6286,7 +6295,7 @@
         <v>200</v>
       </c>
       <c r="F189" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G189" s="2" t="s">
         <v>50</v>
@@ -6296,7 +6305,7 @@
       </c>
       <c r="I189" s="2"/>
       <c r="K189" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="190" spans="1:12" x14ac:dyDescent="0.25">
@@ -6354,7 +6363,7 @@
       </c>
       <c r="I192" s="5"/>
       <c r="K192" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="193" spans="2:12" x14ac:dyDescent="0.25">
@@ -6371,7 +6380,7 @@
         <v>59</v>
       </c>
       <c r="K193" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="194" spans="2:12" x14ac:dyDescent="0.25">
@@ -6412,7 +6421,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K195" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="196" spans="2:12" x14ac:dyDescent="0.25">
@@ -6420,7 +6429,7 @@
         <v>211</v>
       </c>
       <c r="F196" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G196" s="2" t="s">
         <v>50</v>
@@ -6433,7 +6442,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K196" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="197" spans="2:12" x14ac:dyDescent="0.25">
@@ -6470,7 +6479,7 @@
         <v>255</v>
       </c>
       <c r="F198" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G198" s="2" t="s">
         <v>50</v>
@@ -6480,7 +6489,7 @@
       </c>
       <c r="I198" s="2"/>
       <c r="K198" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="199" spans="2:12" x14ac:dyDescent="0.25">
@@ -6500,7 +6509,7 @@
         <v>58</v>
       </c>
       <c r="K199" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="200" spans="2:12" x14ac:dyDescent="0.25">
@@ -6534,7 +6543,7 @@
         <v>59</v>
       </c>
       <c r="K201" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="202" spans="2:12" x14ac:dyDescent="0.25">
@@ -6565,7 +6574,7 @@
         <v>200</v>
       </c>
       <c r="F203" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G203" s="2" t="s">
         <v>50</v>
@@ -6578,7 +6587,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K203" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="204" spans="2:12" x14ac:dyDescent="0.25">
@@ -6586,7 +6595,7 @@
         <v>211</v>
       </c>
       <c r="F204" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G204" s="2" t="s">
         <v>50</v>
@@ -6599,7 +6608,7 @@
         <v>OMOP Systemic Therapy Procedure</v>
       </c>
       <c r="K204" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="205" spans="2:12" x14ac:dyDescent="0.25">
@@ -6633,7 +6642,7 @@
         <v>543</v>
       </c>
       <c r="E206" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F206" s="2" t="s">
         <v>154</v>
@@ -6646,7 +6655,7 @@
       </c>
       <c r="I206" s="10"/>
       <c r="K206" s="2" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="207" spans="2:12" x14ac:dyDescent="0.25">
@@ -6658,7 +6667,7 @@
         <v>285</v>
       </c>
       <c r="F207" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G207" s="2" t="s">
         <v>50</v>
@@ -6667,7 +6676,7 @@
         <v>21</v>
       </c>
       <c r="K207" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="208" spans="2:12" x14ac:dyDescent="0.25">
@@ -6707,10 +6716,10 @@
         <v>62</v>
       </c>
       <c r="J209" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="K209" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="210" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
@@ -6721,7 +6730,7 @@
         <v>292</v>
       </c>
       <c r="F210" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="G210" s="2" t="s">
         <v>57</v>
@@ -6747,7 +6756,7 @@
         <v>59</v>
       </c>
       <c r="K211" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="212" spans="2:12" x14ac:dyDescent="0.25">
@@ -6767,7 +6776,7 @@
         <v>60</v>
       </c>
       <c r="K212" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="213" spans="2:12" x14ac:dyDescent="0.25">
@@ -6815,7 +6824,7 @@
         <v>200</v>
       </c>
       <c r="F215" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G215" s="2" t="s">
         <v>50</v>
@@ -6828,7 +6837,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K215" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="216" spans="2:12" x14ac:dyDescent="0.25">
@@ -6836,7 +6845,7 @@
         <v>211</v>
       </c>
       <c r="F216" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G216" s="2" t="s">
         <v>50</v>
@@ -6849,7 +6858,7 @@
         <v>OMOP Systemic Therapy Dose Given Drug Exposure</v>
       </c>
       <c r="K216" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="217" spans="2:12" x14ac:dyDescent="0.25">
@@ -6886,7 +6895,7 @@
         <v>285</v>
       </c>
       <c r="F218" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G218" s="2" t="s">
         <v>50</v>
@@ -6895,7 +6904,7 @@
         <v>21</v>
       </c>
       <c r="K218" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="219" spans="2:12" x14ac:dyDescent="0.25">
@@ -6935,10 +6944,10 @@
         <v>62</v>
       </c>
       <c r="J220" s="2" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="K220" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="221" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
@@ -6949,7 +6958,7 @@
         <v>292</v>
       </c>
       <c r="F221" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="G221" s="2" t="s">
         <v>57</v>
@@ -6975,7 +6984,7 @@
         <v>59</v>
       </c>
       <c r="K222" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="223" spans="2:12" x14ac:dyDescent="0.25">
@@ -6995,7 +7004,7 @@
         <v>60</v>
       </c>
       <c r="K223" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="224" spans="2:12" x14ac:dyDescent="0.25">
@@ -7043,7 +7052,7 @@
         <v>200</v>
       </c>
       <c r="F226" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G226" s="2" t="s">
         <v>50</v>
@@ -7056,7 +7065,7 @@
         <v>OMOP Systemic Therapy Episode</v>
       </c>
       <c r="K226" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="227" spans="1:12" x14ac:dyDescent="0.25">
@@ -7064,7 +7073,7 @@
         <v>211</v>
       </c>
       <c r="F227" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G227" s="2" t="s">
         <v>50</v>
@@ -7077,7 +7086,7 @@
         <v>OMOP Systemic Therapy Dose Prescribed Drug Exposure</v>
       </c>
       <c r="K227" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="228" spans="1:12" x14ac:dyDescent="0.25">
@@ -7128,7 +7137,7 @@
         <v>200</v>
       </c>
       <c r="F230" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G230" s="2" t="s">
         <v>50</v>
@@ -7137,7 +7146,7 @@
         <v>21</v>
       </c>
       <c r="K230" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="231" spans="1:12" x14ac:dyDescent="0.25">
@@ -7195,7 +7204,7 @@
       </c>
       <c r="I233" s="5"/>
       <c r="K233" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="234" spans="1:12" x14ac:dyDescent="0.25">
@@ -7212,10 +7221,10 @@
         <v>133</v>
       </c>
       <c r="I234" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K234" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="235" spans="1:12" ht="27" x14ac:dyDescent="0.25">
@@ -7242,7 +7251,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K235" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="236" spans="1:12" x14ac:dyDescent="0.25">
@@ -7250,7 +7259,7 @@
         <v>211</v>
       </c>
       <c r="F236" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G236" s="2" t="s">
         <v>50</v>
@@ -7263,7 +7272,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K236" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="237" spans="1:12" x14ac:dyDescent="0.25">
@@ -7300,7 +7309,7 @@
         <v>255</v>
       </c>
       <c r="F238" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G238" s="2" t="s">
         <v>50</v>
@@ -7309,7 +7318,7 @@
         <v>21</v>
       </c>
       <c r="K238" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="239" spans="1:12" x14ac:dyDescent="0.25">
@@ -7329,7 +7338,7 @@
         <v>69</v>
       </c>
       <c r="K239" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="240" spans="1:12" x14ac:dyDescent="0.25">
@@ -7363,10 +7372,10 @@
         <v>133</v>
       </c>
       <c r="I241" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K241" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="242" spans="2:12" x14ac:dyDescent="0.25">
@@ -7416,7 +7425,7 @@
         <v>200</v>
       </c>
       <c r="F244" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G244" s="2" t="s">
         <v>50</v>
@@ -7429,7 +7438,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K244" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="245" spans="2:12" x14ac:dyDescent="0.25">
@@ -7437,7 +7446,7 @@
         <v>211</v>
       </c>
       <c r="F245" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G245" s="2" t="s">
         <v>50</v>
@@ -7450,7 +7459,7 @@
         <v>OMOP Radiation Procedure</v>
       </c>
       <c r="K245" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="246" spans="2:12" x14ac:dyDescent="0.25">
@@ -7487,7 +7496,7 @@
         <v>213</v>
       </c>
       <c r="F247" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G247" s="2" t="s">
         <v>50</v>
@@ -7496,7 +7505,7 @@
         <v>21</v>
       </c>
       <c r="K247" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="248" spans="2:12" x14ac:dyDescent="0.25">
@@ -7536,10 +7545,10 @@
         <v>133</v>
       </c>
       <c r="I249" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K249" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="250" spans="2:12" x14ac:dyDescent="0.25">
@@ -7547,7 +7556,7 @@
         <v>149</v>
       </c>
       <c r="F250" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G250" s="2" t="s">
         <v>50</v>
@@ -7560,7 +7569,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K250" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="251" spans="2:12" x14ac:dyDescent="0.25">
@@ -7603,7 +7612,7 @@
         <v>72</v>
       </c>
       <c r="K252" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="253" spans="2:12" x14ac:dyDescent="0.25">
@@ -7643,7 +7652,7 @@
         <v>213</v>
       </c>
       <c r="F254" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G254" s="2" t="s">
         <v>50</v>
@@ -7652,7 +7661,7 @@
         <v>21</v>
       </c>
       <c r="K254" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="255" spans="2:12" x14ac:dyDescent="0.25">
@@ -7690,10 +7699,10 @@
         <v>133</v>
       </c>
       <c r="I256" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K256" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="257" spans="2:12" x14ac:dyDescent="0.25">
@@ -7701,7 +7710,7 @@
         <v>149</v>
       </c>
       <c r="F257" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G257" s="2" t="s">
         <v>50</v>
@@ -7714,7 +7723,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K257" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="258" spans="2:12" x14ac:dyDescent="0.25">
@@ -7757,7 +7766,7 @@
         <v>71</v>
       </c>
       <c r="K259" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="260" spans="2:12" ht="27" x14ac:dyDescent="0.25">
@@ -7771,7 +7780,7 @@
         <v>172</v>
       </c>
       <c r="F260" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G260" s="2" t="s">
         <v>50</v>
@@ -7780,7 +7789,7 @@
         <v>21</v>
       </c>
       <c r="K260" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="261" spans="2:12" x14ac:dyDescent="0.25">
@@ -7820,10 +7829,10 @@
         <v>133</v>
       </c>
       <c r="I262" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K262" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="263" spans="2:12" x14ac:dyDescent="0.25">
@@ -7831,7 +7840,7 @@
         <v>228</v>
       </c>
       <c r="F263" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G263" s="2" t="s">
         <v>50</v>
@@ -7844,7 +7853,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K263" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="264" spans="2:12" x14ac:dyDescent="0.25">
@@ -7887,7 +7896,7 @@
         <v>73</v>
       </c>
       <c r="K265" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="266" spans="2:12" x14ac:dyDescent="0.25">
@@ -7918,7 +7927,7 @@
         <v>255</v>
       </c>
       <c r="F267" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G267" s="2" t="s">
         <v>50</v>
@@ -7927,7 +7936,7 @@
         <v>21</v>
       </c>
       <c r="K267" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="268" spans="2:12" x14ac:dyDescent="0.25">
@@ -7967,10 +7976,10 @@
         <v>133</v>
       </c>
       <c r="I269" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K269" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="270" spans="2:12" x14ac:dyDescent="0.25">
@@ -7987,7 +7996,7 @@
         <v>74</v>
       </c>
       <c r="K270" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="271" spans="2:12" x14ac:dyDescent="0.25">
@@ -8015,7 +8024,7 @@
         <v>200</v>
       </c>
       <c r="F272" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G272" s="2" t="s">
         <v>50</v>
@@ -8028,7 +8037,7 @@
         <v>OMOP Radiation Episode</v>
       </c>
       <c r="K272" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="273" spans="1:12" x14ac:dyDescent="0.25">
@@ -8036,7 +8045,7 @@
         <v>211</v>
       </c>
       <c r="F273" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G273" s="2" t="s">
         <v>50</v>
@@ -8049,7 +8058,7 @@
         <v>OMOP Radiation Boost Procedure</v>
       </c>
       <c r="K273" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="274" spans="1:12" x14ac:dyDescent="0.25">
@@ -8089,7 +8098,7 @@
         <v>133</v>
       </c>
       <c r="F275" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G275" s="2" t="s">
         <v>75</v>
@@ -8106,7 +8115,7 @@
         <v>200</v>
       </c>
       <c r="F276" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G276" s="2" t="s">
         <v>50</v>
@@ -8115,7 +8124,7 @@
         <v>21</v>
       </c>
       <c r="K276" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="277" spans="1:12" x14ac:dyDescent="0.25">
@@ -8173,10 +8182,10 @@
       </c>
       <c r="I279" s="5"/>
       <c r="J279" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="K279" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="280" spans="1:12" x14ac:dyDescent="0.25">
@@ -8193,10 +8202,10 @@
         <v>133</v>
       </c>
       <c r="I280" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K280" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="281" spans="1:12" ht="27" x14ac:dyDescent="0.25">
@@ -8223,7 +8232,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K281" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="282" spans="1:12" x14ac:dyDescent="0.25">
@@ -8231,7 +8240,7 @@
         <v>211</v>
       </c>
       <c r="F282" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G282" s="2" t="s">
         <v>50</v>
@@ -8244,7 +8253,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K282" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="283" spans="1:12" x14ac:dyDescent="0.25">
@@ -8281,7 +8290,7 @@
         <v>255</v>
       </c>
       <c r="F284" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G284" s="2" t="s">
         <v>50</v>
@@ -8290,7 +8299,7 @@
         <v>21</v>
       </c>
       <c r="K284" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="285" spans="1:12" x14ac:dyDescent="0.25">
@@ -8311,10 +8320,10 @@
       </c>
       <c r="I285" s="5"/>
       <c r="J285" s="2" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="K285" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="286" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
@@ -8325,7 +8334,7 @@
         <v>258</v>
       </c>
       <c r="F286" s="2" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="G286" s="2" t="s">
         <v>75</v>
@@ -8348,10 +8357,10 @@
         <v>133</v>
       </c>
       <c r="I287" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K287" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="288" spans="1:12" ht="27" x14ac:dyDescent="0.25">
@@ -8365,7 +8374,7 @@
         <v>200</v>
       </c>
       <c r="F288" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G288" s="2" t="s">
         <v>50</v>
@@ -8378,7 +8387,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K288" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="289" spans="2:12" x14ac:dyDescent="0.25">
@@ -8386,7 +8395,7 @@
         <v>211</v>
       </c>
       <c r="F289" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G289" s="2" t="s">
         <v>50</v>
@@ -8399,7 +8408,7 @@
         <v>OMOP Surgery Procedure</v>
       </c>
       <c r="K289" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="290" spans="2:12" x14ac:dyDescent="0.25">
@@ -8436,7 +8445,7 @@
         <v>213</v>
       </c>
       <c r="F291" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G291" s="2" t="s">
         <v>50</v>
@@ -8445,7 +8454,7 @@
         <v>21</v>
       </c>
       <c r="K291" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="292" spans="2:12" x14ac:dyDescent="0.25">
@@ -8480,10 +8489,10 @@
         <v>133</v>
       </c>
       <c r="I293" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K293" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="294" spans="2:12" x14ac:dyDescent="0.25">
@@ -8491,7 +8500,7 @@
         <v>149</v>
       </c>
       <c r="F294" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G294" s="2" t="s">
         <v>50</v>
@@ -8504,7 +8513,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K294" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="295" spans="2:12" x14ac:dyDescent="0.25">
@@ -8547,7 +8556,7 @@
         <v>80</v>
       </c>
       <c r="K296" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="297" spans="2:12" x14ac:dyDescent="0.25">
@@ -8584,7 +8593,7 @@
         <v>213</v>
       </c>
       <c r="F298" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G298" s="2" t="s">
         <v>50</v>
@@ -8593,7 +8602,7 @@
         <v>21</v>
       </c>
       <c r="K298" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="299" spans="2:12" x14ac:dyDescent="0.25">
@@ -8628,10 +8637,10 @@
         <v>133</v>
       </c>
       <c r="I300" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K300" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="301" spans="2:12" x14ac:dyDescent="0.25">
@@ -8639,7 +8648,7 @@
         <v>149</v>
       </c>
       <c r="F301" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G301" s="2" t="s">
         <v>50</v>
@@ -8652,7 +8661,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K301" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="302" spans="2:12" x14ac:dyDescent="0.25">
@@ -8695,7 +8704,7 @@
         <v>81</v>
       </c>
       <c r="K303" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="304" spans="2:12" x14ac:dyDescent="0.25">
@@ -8732,7 +8741,7 @@
         <v>213</v>
       </c>
       <c r="F305" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G305" s="2" t="s">
         <v>50</v>
@@ -8741,7 +8750,7 @@
         <v>21</v>
       </c>
       <c r="K305" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="306" spans="2:12" x14ac:dyDescent="0.25">
@@ -8776,10 +8785,10 @@
         <v>133</v>
       </c>
       <c r="I307" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K307" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="308" spans="2:12" x14ac:dyDescent="0.25">
@@ -8787,7 +8796,7 @@
         <v>149</v>
       </c>
       <c r="F308" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G308" s="2" t="s">
         <v>50</v>
@@ -8800,7 +8809,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K308" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="309" spans="2:12" x14ac:dyDescent="0.25">
@@ -8843,7 +8852,7 @@
         <v>82</v>
       </c>
       <c r="K310" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="311" spans="2:12" x14ac:dyDescent="0.25">
@@ -8880,7 +8889,7 @@
         <v>172</v>
       </c>
       <c r="F312" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G312" s="2" t="s">
         <v>50</v>
@@ -8889,7 +8898,7 @@
         <v>21</v>
       </c>
       <c r="K312" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="313" spans="2:12" x14ac:dyDescent="0.25">
@@ -8929,10 +8938,10 @@
         <v>133</v>
       </c>
       <c r="I314" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K314" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="315" spans="2:12" x14ac:dyDescent="0.25">
@@ -8940,7 +8949,7 @@
         <v>228</v>
       </c>
       <c r="F315" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G315" s="2" t="s">
         <v>50</v>
@@ -8953,7 +8962,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K315" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="316" spans="2:12" x14ac:dyDescent="0.25">
@@ -8999,7 +9008,7 @@
         <v>531</v>
       </c>
       <c r="K317" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="318" spans="2:12" x14ac:dyDescent="0.25">
@@ -9030,7 +9039,7 @@
         <v>172</v>
       </c>
       <c r="F319" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G319" s="2" t="s">
         <v>50</v>
@@ -9039,7 +9048,7 @@
         <v>21</v>
       </c>
       <c r="K319" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="320" spans="2:12" x14ac:dyDescent="0.25">
@@ -9079,10 +9088,10 @@
         <v>133</v>
       </c>
       <c r="I321" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K321" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="322" spans="2:12" x14ac:dyDescent="0.25">
@@ -9090,7 +9099,7 @@
         <v>228</v>
       </c>
       <c r="F322" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G322" s="2" t="s">
         <v>50</v>
@@ -9103,7 +9112,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K322" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="323" spans="2:12" x14ac:dyDescent="0.25">
@@ -9146,7 +9155,7 @@
         <v>83</v>
       </c>
       <c r="K324" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="325" spans="2:12" x14ac:dyDescent="0.25">
@@ -9177,7 +9186,7 @@
         <v>172</v>
       </c>
       <c r="F326" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G326" s="2" t="s">
         <v>50</v>
@@ -9186,7 +9195,7 @@
         <v>21</v>
       </c>
       <c r="K326" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="327" spans="2:12" x14ac:dyDescent="0.25">
@@ -9226,10 +9235,10 @@
         <v>133</v>
       </c>
       <c r="I328" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K328" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="329" spans="2:12" x14ac:dyDescent="0.25">
@@ -9237,7 +9246,7 @@
         <v>228</v>
       </c>
       <c r="F329" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G329" s="2" t="s">
         <v>50</v>
@@ -9250,7 +9259,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K329" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="330" spans="2:12" x14ac:dyDescent="0.25">
@@ -9293,7 +9302,7 @@
         <v>79</v>
       </c>
       <c r="K331" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="332" spans="2:12" x14ac:dyDescent="0.25">
@@ -9324,7 +9333,7 @@
         <v>172</v>
       </c>
       <c r="F333" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G333" s="2" t="s">
         <v>50</v>
@@ -9333,7 +9342,7 @@
         <v>21</v>
       </c>
       <c r="K333" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="334" spans="2:12" x14ac:dyDescent="0.25">
@@ -9373,10 +9382,10 @@
         <v>133</v>
       </c>
       <c r="I335" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K335" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="336" spans="2:12" x14ac:dyDescent="0.25">
@@ -9384,7 +9393,7 @@
         <v>228</v>
       </c>
       <c r="F336" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G336" s="2" t="s">
         <v>50</v>
@@ -9397,7 +9406,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K336" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="337" spans="2:12" x14ac:dyDescent="0.25">
@@ -9440,7 +9449,7 @@
         <v>84</v>
       </c>
       <c r="K338" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="339" spans="2:12" x14ac:dyDescent="0.25">
@@ -9471,7 +9480,7 @@
         <v>172</v>
       </c>
       <c r="F340" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G340" s="2" t="s">
         <v>50</v>
@@ -9480,7 +9489,7 @@
         <v>21</v>
       </c>
       <c r="K340" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="341" spans="2:12" x14ac:dyDescent="0.25">
@@ -9520,10 +9529,10 @@
         <v>133</v>
       </c>
       <c r="I342" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K342" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="343" spans="2:12" x14ac:dyDescent="0.25">
@@ -9531,7 +9540,7 @@
         <v>228</v>
       </c>
       <c r="F343" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G343" s="2" t="s">
         <v>50</v>
@@ -9544,7 +9553,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K343" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="344" spans="2:12" x14ac:dyDescent="0.25">
@@ -9587,7 +9596,7 @@
         <v>88</v>
       </c>
       <c r="K345" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="346" spans="2:12" x14ac:dyDescent="0.25">
@@ -9618,7 +9627,7 @@
         <v>172</v>
       </c>
       <c r="F347" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G347" s="2" t="s">
         <v>50</v>
@@ -9627,7 +9636,7 @@
         <v>21</v>
       </c>
       <c r="K347" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="348" spans="2:12" x14ac:dyDescent="0.25">
@@ -9667,10 +9676,10 @@
         <v>133</v>
       </c>
       <c r="I349" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K349" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="350" spans="2:12" x14ac:dyDescent="0.25">
@@ -9678,7 +9687,7 @@
         <v>228</v>
       </c>
       <c r="F350" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G350" s="2" t="s">
         <v>50</v>
@@ -9691,7 +9700,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K350" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="351" spans="2:12" x14ac:dyDescent="0.25">
@@ -9734,10 +9743,10 @@
         <v>89</v>
       </c>
       <c r="K352" s="2" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="353" spans="2:12" x14ac:dyDescent="0.25">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="353" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C353" s="2" t="s">
         <v>377</v>
       </c>
@@ -9754,7 +9763,10 @@
         <v>89</v>
       </c>
     </row>
-    <row r="354" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A354" s="5" t="s">
+        <v>621</v>
+      </c>
       <c r="B354" s="3" t="s">
         <v>469</v>
       </c>
@@ -9765,7 +9777,7 @@
         <v>172</v>
       </c>
       <c r="F354" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G354" s="2" t="s">
         <v>50</v>
@@ -9774,10 +9786,10 @@
         <v>21</v>
       </c>
       <c r="K354" s="2" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="355" spans="2:12" x14ac:dyDescent="0.25">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="355" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E355" s="2" t="s">
         <v>173</v>
       </c>
@@ -9800,7 +9812,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="356" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E356" s="2" t="s">
         <v>135</v>
       </c>
@@ -9814,18 +9826,18 @@
         <v>133</v>
       </c>
       <c r="I356" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K356" s="2" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="357" spans="2:12" x14ac:dyDescent="0.25">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="357" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E357" s="2" t="s">
         <v>228</v>
       </c>
       <c r="F357" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G357" s="2" t="s">
         <v>50</v>
@@ -9838,10 +9850,10 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K357" s="2" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="358" spans="2:12" x14ac:dyDescent="0.25">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="358" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E358" s="2" t="s">
         <v>229</v>
       </c>
@@ -9864,7 +9876,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="359" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C359" s="2" t="s">
         <v>358</v>
       </c>
@@ -9872,19 +9884,16 @@
         <v>176</v>
       </c>
       <c r="F359" s="2" t="s">
-        <v>132</v>
+        <v>618</v>
       </c>
       <c r="G359" s="2" t="s">
-        <v>133</v>
+        <v>75</v>
       </c>
       <c r="H359" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="I359" s="3" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="360" spans="2:12" x14ac:dyDescent="0.25">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="360" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C360" s="2" t="s">
         <v>359</v>
       </c>
@@ -9892,19 +9901,16 @@
         <v>178</v>
       </c>
       <c r="F360" s="2" t="s">
-        <v>550</v>
+        <v>611</v>
       </c>
       <c r="G360" s="2" t="s">
-        <v>75</v>
+        <v>133</v>
       </c>
       <c r="H360" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="K360" s="2" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="361" spans="2:12" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="361" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E361" s="2" t="s">
         <v>275</v>
       </c>
@@ -9927,7 +9933,10 @@
         <v>361</v>
       </c>
     </row>
-    <row r="362" spans="2:12" ht="40.5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A362" s="5" t="s">
+        <v>622</v>
+      </c>
       <c r="B362" s="3" t="s">
         <v>470</v>
       </c>
@@ -9938,7 +9947,7 @@
         <v>172</v>
       </c>
       <c r="F362" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G362" s="2" t="s">
         <v>50</v>
@@ -9947,10 +9956,10 @@
         <v>21</v>
       </c>
       <c r="K362" s="2" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="363" spans="2:12" x14ac:dyDescent="0.25">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="363" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E363" s="2" t="s">
         <v>173</v>
       </c>
@@ -9973,7 +9982,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="364" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E364" s="2" t="s">
         <v>135</v>
       </c>
@@ -9987,18 +9996,18 @@
         <v>133</v>
       </c>
       <c r="I364" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K364" s="2" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="365" spans="2:12" x14ac:dyDescent="0.25">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="365" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E365" s="2" t="s">
         <v>228</v>
       </c>
       <c r="F365" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G365" s="2" t="s">
         <v>50</v>
@@ -10011,10 +10020,10 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K365" s="2" t="s">
-        <v>562</v>
-      </c>
-    </row>
-    <row r="366" spans="2:12" x14ac:dyDescent="0.25">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="366" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E366" s="2" t="s">
         <v>229</v>
       </c>
@@ -10037,7 +10046,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="367" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C367" s="2" t="s">
         <v>362</v>
       </c>
@@ -10045,19 +10054,16 @@
         <v>176</v>
       </c>
       <c r="F367" s="2" t="s">
-        <v>132</v>
+        <v>618</v>
       </c>
       <c r="G367" s="2" t="s">
-        <v>133</v>
+        <v>75</v>
       </c>
       <c r="H367" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="I367" s="3" t="s">
-        <v>549</v>
-      </c>
-    </row>
-    <row r="368" spans="2:12" x14ac:dyDescent="0.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="368" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C368" s="2" t="s">
         <v>363</v>
       </c>
@@ -10065,16 +10071,13 @@
         <v>178</v>
       </c>
       <c r="F368" s="2" t="s">
-        <v>550</v>
+        <v>611</v>
       </c>
       <c r="G368" s="2" t="s">
-        <v>75</v>
+        <v>133</v>
       </c>
       <c r="H368" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="K368" s="2" t="s">
-        <v>562</v>
+        <v>133</v>
       </c>
     </row>
     <row r="369" spans="1:12" x14ac:dyDescent="0.25">
@@ -10101,6 +10104,9 @@
       </c>
     </row>
     <row r="370" spans="1:12" ht="40.5" x14ac:dyDescent="0.25">
+      <c r="A370" s="5" t="s">
+        <v>623</v>
+      </c>
       <c r="B370" s="3" t="s">
         <v>471</v>
       </c>
@@ -10111,7 +10117,7 @@
         <v>172</v>
       </c>
       <c r="F370" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G370" s="2" t="s">
         <v>50</v>
@@ -10120,7 +10126,7 @@
         <v>21</v>
       </c>
       <c r="K370" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="371" spans="1:12" x14ac:dyDescent="0.25">
@@ -10160,10 +10166,10 @@
         <v>133</v>
       </c>
       <c r="I372" s="3" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="K372" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="373" spans="1:12" x14ac:dyDescent="0.25">
@@ -10171,7 +10177,7 @@
         <v>228</v>
       </c>
       <c r="F373" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G373" s="2" t="s">
         <v>50</v>
@@ -10184,7 +10190,7 @@
         <v>OMOP Surgery Episode</v>
       </c>
       <c r="K373" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="374" spans="1:12" x14ac:dyDescent="0.25">
@@ -10218,16 +10224,13 @@
         <v>176</v>
       </c>
       <c r="F375" s="2" t="s">
-        <v>132</v>
+        <v>618</v>
       </c>
       <c r="G375" s="2" t="s">
-        <v>133</v>
+        <v>75</v>
       </c>
       <c r="H375" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="I375" s="3" t="s">
-        <v>549</v>
+        <v>87</v>
       </c>
     </row>
     <row r="376" spans="1:12" x14ac:dyDescent="0.25">
@@ -10238,16 +10241,13 @@
         <v>178</v>
       </c>
       <c r="F376" s="2" t="s">
-        <v>550</v>
+        <v>611</v>
       </c>
       <c r="G376" s="2" t="s">
-        <v>75</v>
+        <v>133</v>
       </c>
       <c r="H376" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="K376" s="2" t="s">
-        <v>562</v>
+        <v>133</v>
       </c>
     </row>
     <row r="377" spans="1:12" x14ac:dyDescent="0.25">
@@ -10284,7 +10284,7 @@
         <v>543</v>
       </c>
       <c r="E378" s="2" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="F378" s="2" t="s">
         <v>154</v>
@@ -10296,7 +10296,7 @@
         <v>3</v>
       </c>
       <c r="K378" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="379" spans="1:12" x14ac:dyDescent="0.25">
@@ -10322,25 +10322,25 @@
       <c r="A380" s="2"/>
       <c r="B380" s="2"/>
       <c r="E380" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="F380" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G380" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H380" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="I380" s="3" t="s">
         <v>596</v>
-      </c>
-      <c r="F380" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G380" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H380" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="I380" s="3" t="s">
-        <v>597</v>
       </c>
       <c r="J380" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L380" s="2" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="381" spans="1:12" x14ac:dyDescent="0.25">
@@ -10360,7 +10360,7 @@
         <v>22</v>
       </c>
       <c r="K381" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="382" spans="1:12" x14ac:dyDescent="0.25">
@@ -10420,7 +10420,7 @@
         <v>3</v>
       </c>
       <c r="K384" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="385" spans="2:12" x14ac:dyDescent="0.25">
@@ -10460,7 +10460,7 @@
         <v>22</v>
       </c>
       <c r="K386" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="387" spans="2:12" x14ac:dyDescent="0.25">
@@ -10481,7 +10481,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K387" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="388" spans="2:12" x14ac:dyDescent="0.25">
@@ -10527,7 +10527,7 @@
         <v>531</v>
       </c>
       <c r="K389" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="390" spans="2:12" x14ac:dyDescent="0.25">
@@ -10567,7 +10567,7 @@
         <v>3</v>
       </c>
       <c r="K391" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="392" spans="2:12" x14ac:dyDescent="0.25">
@@ -10584,7 +10584,7 @@
         <v>133</v>
       </c>
       <c r="I392" s="3" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="J392" s="2" t="s">
         <v>174</v>
@@ -10607,7 +10607,7 @@
         <v>22</v>
       </c>
       <c r="K393" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="394" spans="2:12" x14ac:dyDescent="0.25">
@@ -10628,7 +10628,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K394" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="395" spans="2:12" x14ac:dyDescent="0.25">
@@ -10671,7 +10671,7 @@
         <v>29</v>
       </c>
       <c r="K396" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="397" spans="2:12" x14ac:dyDescent="0.25">
@@ -10745,7 +10745,7 @@
         <v>3</v>
       </c>
       <c r="K400" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="401" spans="2:12" x14ac:dyDescent="0.25">
@@ -10785,7 +10785,7 @@
         <v>22</v>
       </c>
       <c r="K402" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="403" spans="2:12" x14ac:dyDescent="0.25">
@@ -10806,7 +10806,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K403" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="404" spans="2:12" x14ac:dyDescent="0.25">
@@ -10849,7 +10849,7 @@
         <v>24</v>
       </c>
       <c r="K405" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="406" spans="2:12" x14ac:dyDescent="0.25">
@@ -10889,7 +10889,7 @@
         <v>3</v>
       </c>
       <c r="K407" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="408" spans="2:12" x14ac:dyDescent="0.25">
@@ -10929,7 +10929,7 @@
         <v>22</v>
       </c>
       <c r="K409" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="410" spans="2:12" x14ac:dyDescent="0.25">
@@ -10950,7 +10950,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K410" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="411" spans="2:12" x14ac:dyDescent="0.25">
@@ -10993,7 +10993,7 @@
         <v>33</v>
       </c>
       <c r="K412" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="413" spans="2:12" x14ac:dyDescent="0.25">
@@ -11033,7 +11033,7 @@
         <v>3</v>
       </c>
       <c r="K414" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="415" spans="2:12" x14ac:dyDescent="0.25">
@@ -11073,7 +11073,7 @@
         <v>22</v>
       </c>
       <c r="K416" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="417" spans="1:12" x14ac:dyDescent="0.25">
@@ -11094,7 +11094,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K417" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="418" spans="1:12" x14ac:dyDescent="0.25">
@@ -11137,7 +11137,7 @@
         <v>32</v>
       </c>
       <c r="K419" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="420" spans="1:12" x14ac:dyDescent="0.25">
@@ -11181,7 +11181,7 @@
         <v>OMOP Primary Dx Episode</v>
       </c>
       <c r="K421" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="422" spans="1:12" x14ac:dyDescent="0.25">
@@ -11202,7 +11202,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K422" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="423" spans="1:12" x14ac:dyDescent="0.25">
@@ -11252,7 +11252,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K424" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="425" spans="1:12" x14ac:dyDescent="0.25">
@@ -11273,7 +11273,7 @@
         <v>OMOP Specimen</v>
       </c>
       <c r="K425" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="426" spans="1:12" x14ac:dyDescent="0.25">
@@ -11336,10 +11336,10 @@
     </row>
     <row r="431" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A431" s="5" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B431" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D431" s="2" t="s">
         <v>543</v>
@@ -11348,7 +11348,7 @@
         <v>133</v>
       </c>
       <c r="F431" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G431" s="2" t="s">
         <v>90</v>
@@ -11361,10 +11361,10 @@
       <c r="A432" s="2"/>
       <c r="B432" s="2"/>
       <c r="D432" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E432" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F432" s="2" t="s">
         <v>153</v>
@@ -11376,35 +11376,35 @@
         <v>91</v>
       </c>
       <c r="K432" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="433" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E433" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="F433" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G433" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H433" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="I433" s="3" t="s">
         <v>568</v>
       </c>
-      <c r="F433" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G433" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H433" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="I433" s="3" t="s">
+      <c r="J433" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="J433" s="2" t="s">
+      <c r="L433" s="2" t="s">
         <v>570</v>
-      </c>
-      <c r="L433" s="2" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="434" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E434" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F434" s="2" t="s">
         <v>183</v>
@@ -11416,12 +11416,12 @@
         <v>92</v>
       </c>
       <c r="K434" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="435" spans="2:12" x14ac:dyDescent="0.25">
       <c r="E435" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F435" s="2" t="s">
         <v>183</v>
@@ -11434,12 +11434,12 @@
       </c>
       <c r="I435" s="8"/>
       <c r="K435" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="436" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B436" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D436" s="2" t="s">
         <v>130</v>
@@ -11457,7 +11457,7 @@
         <v>91</v>
       </c>
       <c r="K436" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="437" spans="2:12" x14ac:dyDescent="0.25">
@@ -11474,13 +11474,13 @@
         <v>133</v>
       </c>
       <c r="I437" s="3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="J437" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L437" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="438" spans="2:12" x14ac:dyDescent="0.25">
@@ -11497,7 +11497,7 @@
         <v>95</v>
       </c>
       <c r="K438" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="439" spans="2:12" x14ac:dyDescent="0.25">
@@ -11532,13 +11532,13 @@
         <v>133</v>
       </c>
       <c r="I440" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J440" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L440" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="441" spans="2:12" x14ac:dyDescent="0.25">
@@ -11555,7 +11555,7 @@
         <v>93</v>
       </c>
       <c r="K441" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="442" spans="2:12" x14ac:dyDescent="0.25">
@@ -11574,7 +11574,7 @@
     </row>
     <row r="443" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B443" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D443" s="2" t="s">
         <v>130</v>
@@ -11592,7 +11592,7 @@
         <v>91</v>
       </c>
       <c r="K443" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="444" spans="2:12" x14ac:dyDescent="0.25">
@@ -11609,13 +11609,13 @@
         <v>133</v>
       </c>
       <c r="I444" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="J444" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L444" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="445" spans="2:12" x14ac:dyDescent="0.25">
@@ -11636,7 +11636,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K445" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="446" spans="2:12" x14ac:dyDescent="0.25">
@@ -11653,13 +11653,13 @@
         <v>133</v>
       </c>
       <c r="I446" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J446" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L446" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="447" spans="2:12" x14ac:dyDescent="0.25">
@@ -11676,7 +11676,7 @@
         <v>94</v>
       </c>
       <c r="K447" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="448" spans="2:12" x14ac:dyDescent="0.25">
@@ -11713,7 +11713,7 @@
         <v>91</v>
       </c>
       <c r="K449" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="450" spans="1:12" x14ac:dyDescent="0.25">
@@ -11757,7 +11757,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K451" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="452" spans="1:12" x14ac:dyDescent="0.25">
@@ -11774,13 +11774,13 @@
         <v>133</v>
       </c>
       <c r="I452" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J452" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L452" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="453" spans="1:12" x14ac:dyDescent="0.25">
@@ -11800,7 +11800,7 @@
         <v>531</v>
       </c>
       <c r="K453" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="454" spans="1:12" x14ac:dyDescent="0.25">
@@ -11830,10 +11830,10 @@
     </row>
     <row r="456" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A456" s="5" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B456" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D456" s="2" t="s">
         <v>543</v>
@@ -11842,7 +11842,7 @@
         <v>133</v>
       </c>
       <c r="F456" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G456" s="2" t="s">
         <v>90</v>
@@ -11855,10 +11855,10 @@
       <c r="A457" s="2"/>
       <c r="B457" s="2"/>
       <c r="D457" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E457" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F457" s="2" t="s">
         <v>153</v>
@@ -11870,35 +11870,35 @@
         <v>91</v>
       </c>
       <c r="K457" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="458" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E458" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="F458" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G458" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H458" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="I458" s="3" t="s">
         <v>568</v>
       </c>
-      <c r="F458" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G458" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H458" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="I458" s="3" t="s">
+      <c r="J458" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="J458" s="2" t="s">
+      <c r="L458" s="2" t="s">
         <v>570</v>
-      </c>
-      <c r="L458" s="2" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="459" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E459" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F459" s="2" t="s">
         <v>183</v>
@@ -11910,12 +11910,12 @@
         <v>92</v>
       </c>
       <c r="K459" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="460" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E460" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F460" s="2" t="s">
         <v>183</v>
@@ -11928,12 +11928,12 @@
       </c>
       <c r="I460" s="8"/>
       <c r="K460" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="461" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B461" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D461" s="2" t="s">
         <v>130</v>
@@ -11951,7 +11951,7 @@
         <v>91</v>
       </c>
       <c r="K461" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="462" spans="1:12" x14ac:dyDescent="0.25">
@@ -11968,13 +11968,13 @@
         <v>133</v>
       </c>
       <c r="I462" s="3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="J462" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L462" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="463" spans="1:12" x14ac:dyDescent="0.25">
@@ -11991,7 +11991,7 @@
         <v>95</v>
       </c>
       <c r="K463" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="464" spans="1:12" x14ac:dyDescent="0.25">
@@ -12026,13 +12026,13 @@
         <v>133</v>
       </c>
       <c r="I465" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J465" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L465" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="466" spans="2:12" x14ac:dyDescent="0.25">
@@ -12049,7 +12049,7 @@
         <v>93</v>
       </c>
       <c r="K466" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="467" spans="2:12" x14ac:dyDescent="0.25">
@@ -12068,7 +12068,7 @@
     </row>
     <row r="468" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B468" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D468" s="2" t="s">
         <v>130</v>
@@ -12086,7 +12086,7 @@
         <v>91</v>
       </c>
       <c r="K468" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="469" spans="2:12" x14ac:dyDescent="0.25">
@@ -12103,13 +12103,13 @@
         <v>133</v>
       </c>
       <c r="I469" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="J469" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L469" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="470" spans="2:12" x14ac:dyDescent="0.25">
@@ -12130,7 +12130,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K470" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="471" spans="2:12" x14ac:dyDescent="0.25">
@@ -12147,13 +12147,13 @@
         <v>133</v>
       </c>
       <c r="I471" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J471" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L471" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="472" spans="2:12" x14ac:dyDescent="0.25">
@@ -12170,7 +12170,7 @@
         <v>94</v>
       </c>
       <c r="K472" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="473" spans="2:12" x14ac:dyDescent="0.25">
@@ -12207,7 +12207,7 @@
         <v>91</v>
       </c>
       <c r="K474" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="475" spans="2:12" x14ac:dyDescent="0.25">
@@ -12251,7 +12251,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K476" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="477" spans="2:12" x14ac:dyDescent="0.25">
@@ -12268,13 +12268,13 @@
         <v>133</v>
       </c>
       <c r="I477" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J477" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L477" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="478" spans="2:12" x14ac:dyDescent="0.25">
@@ -12294,7 +12294,7 @@
         <v>531</v>
       </c>
       <c r="K478" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="479" spans="2:12" x14ac:dyDescent="0.25">
@@ -12313,7 +12313,7 @@
     </row>
     <row r="480" spans="2:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B480" s="3" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="D480" s="2" t="s">
         <v>210</v>
@@ -12335,7 +12335,7 @@
         <v>OMOP Primary Dx Episode</v>
       </c>
       <c r="K480" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="481" spans="1:12" x14ac:dyDescent="0.25">
@@ -12356,7 +12356,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K481" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="482" spans="1:12" x14ac:dyDescent="0.25">
@@ -12373,21 +12373,21 @@
         <v>133</v>
       </c>
       <c r="I482" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J482" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L482" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="483" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A483" s="5" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B483" s="3" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="D483" s="2" t="s">
         <v>543</v>
@@ -12396,7 +12396,7 @@
         <v>133</v>
       </c>
       <c r="F483" s="2" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="G483" s="2" t="s">
         <v>90</v>
@@ -12409,10 +12409,10 @@
       <c r="A484" s="2"/>
       <c r="B484" s="2"/>
       <c r="D484" s="2" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="E484" s="2" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F484" s="2" t="s">
         <v>153</v>
@@ -12424,35 +12424,35 @@
         <v>91</v>
       </c>
       <c r="K484" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="485" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E485" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="F485" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G485" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="H485" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="I485" s="3" t="s">
         <v>568</v>
       </c>
-      <c r="F485" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G485" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H485" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="I485" s="3" t="s">
+      <c r="J485" s="2" t="s">
         <v>569</v>
       </c>
-      <c r="J485" s="2" t="s">
+      <c r="L485" s="2" t="s">
         <v>570</v>
-      </c>
-      <c r="L485" s="2" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="486" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E486" s="2" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="F486" s="2" t="s">
         <v>183</v>
@@ -12464,12 +12464,12 @@
         <v>92</v>
       </c>
       <c r="K486" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="487" spans="1:12" x14ac:dyDescent="0.25">
       <c r="E487" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F487" s="2" t="s">
         <v>183</v>
@@ -12482,12 +12482,12 @@
       </c>
       <c r="I487" s="8"/>
       <c r="K487" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="488" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B488" s="3" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D488" s="2" t="s">
         <v>130</v>
@@ -12505,7 +12505,7 @@
         <v>91</v>
       </c>
       <c r="K488" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="489" spans="1:12" x14ac:dyDescent="0.25">
@@ -12522,13 +12522,13 @@
         <v>133</v>
       </c>
       <c r="I489" s="3" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="J489" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L489" s="2" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="490" spans="1:12" x14ac:dyDescent="0.25">
@@ -12545,7 +12545,7 @@
         <v>95</v>
       </c>
       <c r="K490" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="491" spans="1:12" x14ac:dyDescent="0.25">
@@ -12580,13 +12580,13 @@
         <v>133</v>
       </c>
       <c r="I492" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J492" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L492" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="493" spans="1:12" x14ac:dyDescent="0.25">
@@ -12603,7 +12603,7 @@
         <v>93</v>
       </c>
       <c r="K493" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="494" spans="1:12" x14ac:dyDescent="0.25">
@@ -12622,7 +12622,7 @@
     </row>
     <row r="495" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B495" s="3" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="D495" s="2" t="s">
         <v>130</v>
@@ -12640,7 +12640,7 @@
         <v>91</v>
       </c>
       <c r="K495" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="496" spans="1:12" x14ac:dyDescent="0.25">
@@ -12657,13 +12657,13 @@
         <v>133</v>
       </c>
       <c r="I496" s="3" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="J496" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L496" s="2" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="497" spans="1:12" x14ac:dyDescent="0.25">
@@ -12684,7 +12684,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K497" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="498" spans="1:12" x14ac:dyDescent="0.25">
@@ -12701,13 +12701,13 @@
         <v>133</v>
       </c>
       <c r="I498" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J498" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L498" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="499" spans="1:12" x14ac:dyDescent="0.25">
@@ -12724,7 +12724,7 @@
         <v>94</v>
       </c>
       <c r="K499" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="500" spans="1:12" x14ac:dyDescent="0.25">
@@ -12761,7 +12761,7 @@
         <v>91</v>
       </c>
       <c r="K501" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="502" spans="1:12" x14ac:dyDescent="0.25">
@@ -12805,7 +12805,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K503" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="504" spans="1:12" x14ac:dyDescent="0.25">
@@ -12822,13 +12822,13 @@
         <v>133</v>
       </c>
       <c r="I504" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J504" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L504" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="505" spans="1:12" x14ac:dyDescent="0.25">
@@ -12848,7 +12848,7 @@
         <v>531</v>
       </c>
       <c r="K505" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="506" spans="1:12" x14ac:dyDescent="0.25">
@@ -12867,7 +12867,7 @@
     </row>
     <row r="507" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="B507" s="3" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D507" s="2" t="s">
         <v>210</v>
@@ -12889,7 +12889,7 @@
         <v>OMOP Treatment Episode</v>
       </c>
       <c r="K507" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="508" spans="1:12" x14ac:dyDescent="0.25">
@@ -12910,7 +12910,7 @@
         <v>OMOP Follow Up Visit Occurrence</v>
       </c>
       <c r="K508" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="509" spans="1:12" x14ac:dyDescent="0.25">
@@ -12927,18 +12927,18 @@
         <v>133</v>
       </c>
       <c r="I509" s="3" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="J509" s="2" t="s">
         <v>152</v>
       </c>
       <c r="L509" s="2" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="510" spans="1:12" ht="27" x14ac:dyDescent="0.25">
       <c r="A510" s="5" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="B510" s="3" t="s">
         <v>497</v>
@@ -12950,7 +12950,7 @@
         <v>213</v>
       </c>
       <c r="F510" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G510" s="2" t="s">
         <v>9</v>
@@ -12959,7 +12959,7 @@
         <v>2</v>
       </c>
       <c r="K510" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="511" spans="1:12" x14ac:dyDescent="0.25">
@@ -12999,7 +12999,7 @@
         <v>99</v>
       </c>
       <c r="K512" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="513" spans="2:12" x14ac:dyDescent="0.25">
@@ -13016,7 +13016,7 @@
         <v>100</v>
       </c>
       <c r="K513" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="514" spans="2:12" x14ac:dyDescent="0.25">
@@ -13053,7 +13053,7 @@
         <v>213</v>
       </c>
       <c r="F515" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G515" s="2" t="s">
         <v>9</v>
@@ -13062,7 +13062,7 @@
         <v>2</v>
       </c>
       <c r="K515" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="516" spans="2:12" x14ac:dyDescent="0.25">
@@ -13102,7 +13102,7 @@
         <v>99</v>
       </c>
       <c r="K517" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="518" spans="2:12" x14ac:dyDescent="0.25">
@@ -13119,7 +13119,7 @@
         <v>101</v>
       </c>
       <c r="K518" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="519" spans="2:12" x14ac:dyDescent="0.25">
@@ -13156,7 +13156,7 @@
         <v>213</v>
       </c>
       <c r="F520" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G520" s="2" t="s">
         <v>9</v>
@@ -13165,7 +13165,7 @@
         <v>2</v>
       </c>
       <c r="K520" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="521" spans="2:12" x14ac:dyDescent="0.25">
@@ -13205,7 +13205,7 @@
         <v>99</v>
       </c>
       <c r="K522" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="523" spans="2:12" x14ac:dyDescent="0.25">
@@ -13222,7 +13222,7 @@
         <v>102</v>
       </c>
       <c r="K523" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="524" spans="2:12" x14ac:dyDescent="0.25">
@@ -13259,7 +13259,7 @@
         <v>213</v>
       </c>
       <c r="F525" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G525" s="2" t="s">
         <v>9</v>
@@ -13268,7 +13268,7 @@
         <v>2</v>
       </c>
       <c r="K525" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="526" spans="2:12" x14ac:dyDescent="0.25">
@@ -13308,7 +13308,7 @@
         <v>99</v>
       </c>
       <c r="K527" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="528" spans="2:12" x14ac:dyDescent="0.25">
@@ -13325,7 +13325,7 @@
         <v>103</v>
       </c>
       <c r="K528" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="529" spans="1:12" x14ac:dyDescent="0.25">
@@ -13376,7 +13376,7 @@
         <v>213</v>
       </c>
       <c r="F531" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G531" s="2" t="s">
         <v>9</v>
@@ -13385,7 +13385,7 @@
         <v>2</v>
       </c>
       <c r="K531" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="532" spans="1:12" x14ac:dyDescent="0.25">
@@ -13425,7 +13425,7 @@
         <v>99</v>
       </c>
       <c r="K533" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="534" spans="1:12" x14ac:dyDescent="0.25">
@@ -13442,7 +13442,7 @@
         <v>105</v>
       </c>
       <c r="K534" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="535" spans="1:12" ht="27" x14ac:dyDescent="0.25">
@@ -13456,7 +13456,7 @@
         <v>213</v>
       </c>
       <c r="F535" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G535" s="2" t="s">
         <v>9</v>
@@ -13465,7 +13465,7 @@
         <v>2</v>
       </c>
       <c r="K535" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="536" spans="1:12" x14ac:dyDescent="0.25">
@@ -13505,7 +13505,7 @@
         <v>99</v>
       </c>
       <c r="K537" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="538" spans="1:12" x14ac:dyDescent="0.25">
@@ -13522,7 +13522,7 @@
         <v>106</v>
       </c>
       <c r="K538" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="539" spans="1:12" ht="27" x14ac:dyDescent="0.25">
@@ -13566,7 +13566,7 @@
         <v>172</v>
       </c>
       <c r="F542" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G542" s="2" t="s">
         <v>9</v>
@@ -13575,7 +13575,7 @@
         <v>2</v>
       </c>
       <c r="K542" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="543" spans="1:12" x14ac:dyDescent="0.25">
@@ -13615,7 +13615,7 @@
         <v>118</v>
       </c>
       <c r="K544" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="545" spans="1:12" x14ac:dyDescent="0.25">
@@ -13643,7 +13643,7 @@
         <v>172</v>
       </c>
       <c r="F546" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G546" s="2" t="s">
         <v>9</v>
@@ -13652,7 +13652,7 @@
         <v>2</v>
       </c>
       <c r="K546" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="547" spans="1:12" x14ac:dyDescent="0.25">
@@ -13669,13 +13669,13 @@
         <v>133</v>
       </c>
       <c r="I547" s="3" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="J547" s="2" t="s">
         <v>174</v>
       </c>
       <c r="L547" s="2" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="548" spans="1:12" x14ac:dyDescent="0.25">
@@ -13683,7 +13683,7 @@
         <v>228</v>
       </c>
       <c r="F548" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G548" s="2" t="s">
         <v>9</v>
@@ -13696,7 +13696,7 @@
         <v>OMOP Tobacco Smoking Status Observation</v>
       </c>
       <c r="K548" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="549" spans="1:12" x14ac:dyDescent="0.25">
@@ -13736,10 +13736,13 @@
         <v>120</v>
       </c>
       <c r="K550" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="551" spans="1:12" ht="27" x14ac:dyDescent="0.25">
+      <c r="A551" s="5" t="s">
+        <v>620</v>
+      </c>
       <c r="B551" s="3" t="s">
         <v>504</v>
       </c>
@@ -13750,7 +13753,7 @@
         <v>172</v>
       </c>
       <c r="F551" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G551" s="2" t="s">
         <v>9</v>
@@ -13759,7 +13762,7 @@
         <v>2</v>
       </c>
       <c r="K551" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="552" spans="1:12" x14ac:dyDescent="0.25">
@@ -13790,7 +13793,7 @@
         <v>228</v>
       </c>
       <c r="F553" s="2" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
       <c r="G553" s="2" t="s">
         <v>9</v>
@@ -13803,7 +13806,7 @@
         <v>OMOP Tobacco Smoking Status Observation</v>
       </c>
       <c r="K553" s="2" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="554" spans="1:12" x14ac:dyDescent="0.25">
@@ -13834,16 +13837,13 @@
         <v>176</v>
       </c>
       <c r="F555" s="2" t="s">
-        <v>132</v>
+        <v>618</v>
       </c>
       <c r="G555" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="H555" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="I555" s="3" t="s">
-        <v>549</v>
+        <v>117</v>
+      </c>
+      <c r="H555" s="6" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="556" spans="1:12" x14ac:dyDescent="0.25">
@@ -13851,16 +13851,13 @@
         <v>178</v>
       </c>
       <c r="F556" s="2" t="s">
-        <v>550</v>
+        <v>611</v>
       </c>
       <c r="G556" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="H556" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="K556" s="2" t="s">
-        <v>562</v>
+        <v>133</v>
+      </c>
+      <c r="H556" s="5" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="557" spans="1:12" x14ac:dyDescent="0.25">
@@ -13877,7 +13874,7 @@
         <v>189</v>
       </c>
       <c r="F557" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G557" s="2" t="s">
         <v>9</v>
@@ -13903,7 +13900,7 @@
         <v>193</v>
       </c>
       <c r="K558" s="2" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="559" spans="1:12" x14ac:dyDescent="0.25">
@@ -13925,7 +13922,7 @@
         <v>197</v>
       </c>
       <c r="F560" s="2" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="G560" s="2" t="s">
         <v>110</v>
@@ -13934,7 +13931,7 @@
         <v>113</v>
       </c>
       <c r="K560" s="2" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="561" spans="2:10" x14ac:dyDescent="0.25">
@@ -13976,7 +13973,7 @@
         <v>213</v>
       </c>
       <c r="F563" s="2" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G563" s="2" t="s">
         <v>9</v>
@@ -14076,7 +14073,7 @@
         <v>515</v>
       </c>
       <c r="C569" s="2" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G569" s="12" t="s">
         <v>110</v>

</xml_diff>

<commit_message>
Fixed issue with OMOP Treatment Episode referencing diagnosis id instead of treatment id.
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\serverfiles\projects\dhdp\mohccn-omop-etl\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30804DCB-837B-4224-862C-41F712EDF26A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8B7A6B5-82AD-407C-BB41-794FF427B239}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5774,10 +5774,10 @@
         <v>38</v>
       </c>
       <c r="G166" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="H166" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+      <c r="H166" s="4" t="s">
+        <v>50</v>
       </c>
       <c r="I166" s="2" t="str">
         <f>$B$156</f>

</xml_diff>

<commit_message>
add justin fix, fix concept names
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3534" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3535" uniqueCount="649">
   <si>
     <t xml:space="preserve">Source JSON Level</t>
   </si>
@@ -1491,6 +1491,9 @@
     <t xml:space="preserve">4206020</t>
   </si>
   <si>
+    <t xml:space="preserve">Surgical margin uninvolved by tumor</t>
+  </si>
+  <si>
     <t xml:space="preserve">Surgery - Margin Types Not Involved (Code)</t>
   </si>
   <si>
@@ -1507,6 +1510,9 @@
   </si>
   <si>
     <t xml:space="preserve">4217572</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Surgical margin involvement by tumor cannot be assessed</t>
   </si>
   <si>
     <t xml:space="preserve">Surgery - Margin Types Not Assessable (Code)</t>
@@ -2502,7 +2508,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="24.54"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="47.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="25.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="43.84"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="29.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="22.82"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="33.54"/>
@@ -5960,7 +5966,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B166" s="5" t="s">
         <v>258</v>
       </c>
@@ -5974,10 +5980,10 @@
         <v>38</v>
       </c>
       <c r="G166" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H166" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="I166" s="3" t="str">
         <f aca="false">$B$156</f>
@@ -10233,7 +10239,7 @@
         <v>112</v>
       </c>
       <c r="L368" s="1" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
     </row>
     <row r="369" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10298,7 +10304,7 @@
     </row>
     <row r="372" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C372" s="1" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E372" s="1" t="s">
         <v>115</v>
@@ -10310,12 +10316,12 @@
         <v>386</v>
       </c>
       <c r="H372" s="11" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="373" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C373" s="1" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E373" s="1" t="s">
         <v>118</v>
@@ -10332,10 +10338,10 @@
     </row>
     <row r="374" customFormat="false" ht="36.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="4" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="B374" s="5" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D374" s="1" t="s">
         <v>29</v>
@@ -10370,13 +10376,13 @@
         <v>17</v>
       </c>
       <c r="I375" s="6" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="J375" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L375" s="1" t="s">
-        <v>455</v>
+        <v>471</v>
       </c>
     </row>
     <row r="376" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10441,7 +10447,7 @@
     </row>
     <row r="379" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C379" s="1" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E379" s="1" t="s">
         <v>115</v>
@@ -10453,12 +10459,12 @@
         <v>386</v>
       </c>
       <c r="H379" s="11" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
     </row>
     <row r="380" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C380" s="1" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="E380" s="1" t="s">
         <v>118</v>
@@ -10475,16 +10481,16 @@
     </row>
     <row r="381" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="4" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B381" s="5" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="D381" s="1" t="s">
         <v>64</v>
       </c>
       <c r="E381" s="1" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F381" s="1" t="s">
         <v>21</v>
@@ -10505,7 +10511,7 @@
         <v>25</v>
       </c>
       <c r="E382" s="1" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="F382" s="1" t="s">
         <v>84</v>
@@ -10519,7 +10525,7 @@
     </row>
     <row r="383" s="1" customFormat="true" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E383" s="1" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="F383" s="1" t="s">
         <v>16</v>
@@ -10531,21 +10537,21 @@
         <v>17</v>
       </c>
       <c r="I383" s="6" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="J383" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L383" s="1" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
     </row>
     <row r="384" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C384" s="1" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="E384" s="1" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="F384" s="1" t="s">
         <v>123</v>
@@ -10554,7 +10560,7 @@
         <v>45</v>
       </c>
       <c r="H384" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="K384" s="1" t="s">
         <v>125</v>
@@ -10562,10 +10568,10 @@
     </row>
     <row r="385" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C385" s="1" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="E385" s="1" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="F385" s="1" t="s">
         <v>141</v>
@@ -10574,7 +10580,7 @@
         <v>45</v>
       </c>
       <c r="H385" s="11" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="J385" s="1" t="s">
         <v>418</v>
@@ -10582,10 +10588,10 @@
     </row>
     <row r="386" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C386" s="1" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E386" s="1" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="F386" s="1" t="s">
         <v>21</v>
@@ -10594,12 +10600,12 @@
         <v>45</v>
       </c>
       <c r="H386" s="11" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="387" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E387" s="1" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F387" s="1" t="s">
         <v>21</v>
@@ -10613,7 +10619,7 @@
     </row>
     <row r="388" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B388" s="5" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D388" s="1" t="s">
         <v>14</v>
@@ -10648,13 +10654,13 @@
         <v>17</v>
       </c>
       <c r="I389" s="6" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="J389" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L389" s="1" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="390" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10668,7 +10674,7 @@
         <v>45</v>
       </c>
       <c r="H390" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="K390" s="1" t="s">
         <v>125</v>
@@ -10720,7 +10726,7 @@
     </row>
     <row r="393" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C393" s="1" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="E393" s="1" t="s">
         <v>115</v>
@@ -10732,7 +10738,7 @@
         <v>45</v>
       </c>
       <c r="H393" s="11" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="J393" s="1" t="s">
         <v>418</v>
@@ -10743,7 +10749,7 @@
     </row>
     <row r="394" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C394" s="1" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="E394" s="1" t="s">
         <v>118</v>
@@ -10755,12 +10761,12 @@
         <v>45</v>
       </c>
       <c r="H394" s="11" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="395" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B395" s="5" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D395" s="1" t="s">
         <v>14</v>
@@ -10795,13 +10801,13 @@
         <v>17</v>
       </c>
       <c r="I396" s="6" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="J396" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L396" s="1" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="397" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10815,7 +10821,7 @@
         <v>45</v>
       </c>
       <c r="H397" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="K397" s="1" t="s">
         <v>125</v>
@@ -10867,7 +10873,7 @@
     </row>
     <row r="400" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C400" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="E400" s="1" t="s">
         <v>115</v>
@@ -10879,7 +10885,7 @@
         <v>45</v>
       </c>
       <c r="H400" s="11" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="K400" s="1" t="s">
         <v>92</v>
@@ -10887,7 +10893,7 @@
     </row>
     <row r="401" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C401" s="1" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="E401" s="1" t="s">
         <v>118</v>
@@ -10899,12 +10905,12 @@
         <v>45</v>
       </c>
       <c r="H401" s="11" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="402" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C402" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="E402" s="1" t="s">
         <v>216</v>
@@ -10916,12 +10922,12 @@
         <v>45</v>
       </c>
       <c r="H402" s="11" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="403" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C403" s="1" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="E403" s="1" t="s">
         <v>219</v>
@@ -10933,12 +10939,12 @@
         <v>45</v>
       </c>
       <c r="H403" s="11" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="404" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B404" s="5" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D404" s="1" t="s">
         <v>14</v>
@@ -10973,13 +10979,13 @@
         <v>17</v>
       </c>
       <c r="I405" s="6" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="J405" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L405" s="1" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="406" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10993,7 +10999,7 @@
         <v>45</v>
       </c>
       <c r="H406" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="K406" s="1" t="s">
         <v>125</v>
@@ -11045,7 +11051,7 @@
     </row>
     <row r="409" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C409" s="1" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="E409" s="1" t="s">
         <v>115</v>
@@ -11057,7 +11063,7 @@
         <v>45</v>
       </c>
       <c r="H409" s="11" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="K409" s="1" t="s">
         <v>41</v>
@@ -11065,7 +11071,7 @@
     </row>
     <row r="410" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C410" s="1" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E410" s="1" t="s">
         <v>118</v>
@@ -11077,12 +11083,12 @@
         <v>45</v>
       </c>
       <c r="H410" s="11" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="411" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B411" s="5" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D411" s="1" t="s">
         <v>14</v>
@@ -11117,13 +11123,13 @@
         <v>17</v>
       </c>
       <c r="I412" s="6" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="J412" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L412" s="1" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="413" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11137,7 +11143,7 @@
         <v>45</v>
       </c>
       <c r="H413" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="K413" s="1" t="s">
         <v>125</v>
@@ -11189,7 +11195,7 @@
     </row>
     <row r="416" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C416" s="1" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="E416" s="1" t="s">
         <v>115</v>
@@ -11201,7 +11207,7 @@
         <v>45</v>
       </c>
       <c r="H416" s="11" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="K416" s="1" t="s">
         <v>41</v>
@@ -11209,7 +11215,7 @@
     </row>
     <row r="417" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C417" s="1" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="E417" s="1" t="s">
         <v>118</v>
@@ -11221,12 +11227,12 @@
         <v>45</v>
       </c>
       <c r="H417" s="11" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
     </row>
     <row r="418" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B418" s="5" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="D418" s="1" t="s">
         <v>14</v>
@@ -11261,13 +11267,13 @@
         <v>17</v>
       </c>
       <c r="I419" s="6" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="J419" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L419" s="1" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
     </row>
     <row r="420" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11281,7 +11287,7 @@
         <v>45</v>
       </c>
       <c r="H420" s="11" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="K420" s="1" t="s">
         <v>125</v>
@@ -11333,7 +11339,7 @@
     </row>
     <row r="423" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C423" s="1" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="E423" s="1" t="s">
         <v>115</v>
@@ -11345,7 +11351,7 @@
         <v>45</v>
       </c>
       <c r="H423" s="11" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="K423" s="1" t="s">
         <v>41</v>
@@ -11353,7 +11359,7 @@
     </row>
     <row r="424" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C424" s="1" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="E424" s="1" t="s">
         <v>118</v>
@@ -11365,12 +11371,12 @@
         <v>45</v>
       </c>
       <c r="H424" s="11" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
     </row>
     <row r="425" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B425" s="5" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D425" s="1" t="s">
         <v>163</v>
@@ -11441,7 +11447,7 @@
     </row>
     <row r="428" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B428" s="5" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D428" s="1" t="s">
         <v>163</v>
@@ -11512,13 +11518,13 @@
     </row>
     <row r="431" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B431" s="5" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G431" s="1" t="s">
         <v>45</v>
       </c>
       <c r="H431" s="12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="432" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11526,7 +11532,7 @@
         <v>45</v>
       </c>
       <c r="H432" s="12" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
     </row>
     <row r="433" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11534,7 +11540,7 @@
         <v>45</v>
       </c>
       <c r="H433" s="12" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
     </row>
     <row r="434" customFormat="false" ht="13.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11542,15 +11548,15 @@
         <v>45</v>
       </c>
       <c r="H434" s="12" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
     </row>
     <row r="435" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A435" s="4" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B435" s="5" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D435" s="1" t="s">
         <v>64</v>
@@ -11574,7 +11580,7 @@
         <v>27</v>
       </c>
       <c r="E436" s="1" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F436" s="1" t="s">
         <v>84</v>
@@ -11591,7 +11597,7 @@
     </row>
     <row r="437" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E437" s="1" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F437" s="1" t="s">
         <v>16</v>
@@ -11603,18 +11609,18 @@
         <v>17</v>
       </c>
       <c r="I437" s="6" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="J437" s="1" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="L437" s="1" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="438" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E438" s="1" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F438" s="1" t="s">
         <v>123</v>
@@ -11623,7 +11629,7 @@
         <v>51</v>
       </c>
       <c r="H438" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="K438" s="1" t="s">
         <v>125</v>
@@ -11631,7 +11637,7 @@
     </row>
     <row r="439" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E439" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F439" s="1" t="s">
         <v>123</v>
@@ -11640,7 +11646,7 @@
         <v>51</v>
       </c>
       <c r="H439" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="I439" s="17"/>
       <c r="K439" s="1" t="s">
@@ -11649,7 +11655,7 @@
     </row>
     <row r="440" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B440" s="5" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D440" s="1" t="s">
         <v>14</v>
@@ -11684,13 +11690,13 @@
         <v>17</v>
       </c>
       <c r="I441" s="6" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="J441" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L441" s="1" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="442" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11704,7 +11710,7 @@
         <v>51</v>
       </c>
       <c r="H442" s="11" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="K442" s="1" t="s">
         <v>125</v>
@@ -11762,7 +11768,7 @@
         <v>51</v>
       </c>
       <c r="H445" s="11" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="K445" s="1" t="s">
         <v>41</v>
@@ -11779,12 +11785,12 @@
         <v>51</v>
       </c>
       <c r="H446" s="11" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="447" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B447" s="5" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D447" s="1" t="s">
         <v>14</v>
@@ -11819,13 +11825,13 @@
         <v>17</v>
       </c>
       <c r="I448" s="6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="J448" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L448" s="1" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="449" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11883,7 +11889,7 @@
         <v>51</v>
       </c>
       <c r="H451" s="18" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="K451" s="1" t="s">
         <v>41</v>
@@ -11900,12 +11906,12 @@
         <v>51</v>
       </c>
       <c r="H452" s="18" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="453" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B453" s="5" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D453" s="1" t="s">
         <v>14</v>
@@ -11940,13 +11946,13 @@
         <v>17</v>
       </c>
       <c r="I454" s="6" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="J454" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L454" s="1" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="455" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12004,7 +12010,7 @@
         <v>51</v>
       </c>
       <c r="H457" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="J457" s="1" t="s">
         <v>418</v>
@@ -12024,26 +12030,26 @@
         <v>51</v>
       </c>
       <c r="H458" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="459" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B459" s="5" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="G459" s="1" t="s">
         <v>51</v>
       </c>
       <c r="H459" s="19" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
     <row r="460" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A460" s="4" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B460" s="5" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D460" s="1" t="s">
         <v>64</v>
@@ -12067,7 +12073,7 @@
         <v>27</v>
       </c>
       <c r="E461" s="1" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F461" s="1" t="s">
         <v>84</v>
@@ -12084,7 +12090,7 @@
     </row>
     <row r="462" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E462" s="1" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F462" s="1" t="s">
         <v>16</v>
@@ -12096,18 +12102,18 @@
         <v>17</v>
       </c>
       <c r="I462" s="6" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="J462" s="1" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="L462" s="1" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="463" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E463" s="1" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F463" s="1" t="s">
         <v>123</v>
@@ -12116,7 +12122,7 @@
         <v>51</v>
       </c>
       <c r="H463" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="K463" s="1" t="s">
         <v>125</v>
@@ -12124,7 +12130,7 @@
     </row>
     <row r="464" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E464" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F464" s="1" t="s">
         <v>123</v>
@@ -12133,7 +12139,7 @@
         <v>51</v>
       </c>
       <c r="H464" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="I464" s="17"/>
       <c r="K464" s="1" t="s">
@@ -12142,7 +12148,7 @@
     </row>
     <row r="465" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B465" s="5" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D465" s="1" t="s">
         <v>14</v>
@@ -12177,13 +12183,13 @@
         <v>17</v>
       </c>
       <c r="I466" s="6" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="J466" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L466" s="1" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="467" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12197,7 +12203,7 @@
         <v>51</v>
       </c>
       <c r="H467" s="11" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="K467" s="1" t="s">
         <v>125</v>
@@ -12255,7 +12261,7 @@
         <v>51</v>
       </c>
       <c r="H470" s="11" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="K470" s="1" t="s">
         <v>41</v>
@@ -12272,12 +12278,12 @@
         <v>51</v>
       </c>
       <c r="H471" s="11" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="472" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B472" s="5" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D472" s="1" t="s">
         <v>14</v>
@@ -12312,13 +12318,13 @@
         <v>17</v>
       </c>
       <c r="I473" s="6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="J473" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L473" s="1" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="474" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12376,7 +12382,7 @@
         <v>51</v>
       </c>
       <c r="H476" s="18" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="K476" s="1" t="s">
         <v>41</v>
@@ -12393,12 +12399,12 @@
         <v>51</v>
       </c>
       <c r="H477" s="18" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="478" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B478" s="5" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D478" s="1" t="s">
         <v>14</v>
@@ -12433,13 +12439,13 @@
         <v>17</v>
       </c>
       <c r="I479" s="6" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="J479" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L479" s="1" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="480" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12497,7 +12503,7 @@
         <v>51</v>
       </c>
       <c r="H482" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="J482" s="1" t="s">
         <v>418</v>
@@ -12517,12 +12523,12 @@
         <v>51</v>
       </c>
       <c r="H483" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="484" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B484" s="5" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D484" s="1" t="s">
         <v>163</v>
@@ -12593,10 +12599,10 @@
     </row>
     <row r="487" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A487" s="4" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B487" s="5" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="D487" s="1" t="s">
         <v>64</v>
@@ -12620,7 +12626,7 @@
         <v>27</v>
       </c>
       <c r="E488" s="1" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F488" s="1" t="s">
         <v>84</v>
@@ -12637,7 +12643,7 @@
     </row>
     <row r="489" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E489" s="1" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F489" s="1" t="s">
         <v>16</v>
@@ -12649,18 +12655,18 @@
         <v>17</v>
       </c>
       <c r="I489" s="6" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="J489" s="1" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="L489" s="1" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
     </row>
     <row r="490" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E490" s="1" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="F490" s="1" t="s">
         <v>123</v>
@@ -12669,7 +12675,7 @@
         <v>51</v>
       </c>
       <c r="H490" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="K490" s="1" t="s">
         <v>125</v>
@@ -12677,7 +12683,7 @@
     </row>
     <row r="491" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E491" s="1" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F491" s="1" t="s">
         <v>123</v>
@@ -12686,7 +12692,7 @@
         <v>51</v>
       </c>
       <c r="H491" s="13" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="I491" s="17"/>
       <c r="K491" s="1" t="s">
@@ -12695,7 +12701,7 @@
     </row>
     <row r="492" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B492" s="5" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D492" s="1" t="s">
         <v>14</v>
@@ -12730,13 +12736,13 @@
         <v>17</v>
       </c>
       <c r="I493" s="6" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="J493" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L493" s="1" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
     </row>
     <row r="494" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12750,7 +12756,7 @@
         <v>51</v>
       </c>
       <c r="H494" s="11" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="K494" s="1" t="s">
         <v>125</v>
@@ -12808,7 +12814,7 @@
         <v>51</v>
       </c>
       <c r="H497" s="11" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="K497" s="1" t="s">
         <v>41</v>
@@ -12825,12 +12831,12 @@
         <v>51</v>
       </c>
       <c r="H498" s="11" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
     </row>
     <row r="499" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B499" s="5" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="D499" s="1" t="s">
         <v>14</v>
@@ -12865,13 +12871,13 @@
         <v>17</v>
       </c>
       <c r="I500" s="6" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="J500" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L500" s="1" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
     </row>
     <row r="501" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12929,7 +12935,7 @@
         <v>51</v>
       </c>
       <c r="H503" s="18" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="K503" s="1" t="s">
         <v>41</v>
@@ -12946,12 +12952,12 @@
         <v>51</v>
       </c>
       <c r="H504" s="18" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
     </row>
     <row r="505" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B505" s="5" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D505" s="1" t="s">
         <v>14</v>
@@ -12986,13 +12992,13 @@
         <v>17</v>
       </c>
       <c r="I506" s="6" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="J506" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L506" s="1" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
     </row>
     <row r="507" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13050,7 +13056,7 @@
         <v>51</v>
       </c>
       <c r="H509" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="J509" s="1" t="s">
         <v>418</v>
@@ -13070,12 +13076,12 @@
         <v>51</v>
       </c>
       <c r="H510" s="11" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
     </row>
     <row r="511" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B511" s="5" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="D511" s="1" t="s">
         <v>163</v>
@@ -13146,7 +13152,7 @@
     </row>
     <row r="514" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A514" s="4" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D514" s="1" t="s">
         <v>64</v>
@@ -13158,17 +13164,20 @@
         <v>75</v>
       </c>
       <c r="G514" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H514" s="11" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="I514" s="20"/>
+      <c r="K514" s="1" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="515" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A515" s="0"/>
       <c r="B515" s="5" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="D515" s="1" t="s">
         <v>29</v>
@@ -13203,13 +13212,13 @@
         <v>17</v>
       </c>
       <c r="I516" s="6" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="J516" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L516" s="1" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
     </row>
     <row r="517" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13220,10 +13229,10 @@
         <v>123</v>
       </c>
       <c r="G517" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H517" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K517" s="1" t="s">
         <v>125</v>
@@ -13237,10 +13246,10 @@
         <v>21</v>
       </c>
       <c r="G518" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H518" s="11" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="K518" s="1" t="s">
         <v>41</v>
@@ -13260,18 +13269,18 @@
         <v>17</v>
       </c>
       <c r="I519" s="6" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="J519" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L519" s="1" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="520" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B520" s="5" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="D520" s="1" t="s">
         <v>29</v>
@@ -13306,13 +13315,13 @@
         <v>17</v>
       </c>
       <c r="I521" s="6" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="J521" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L521" s="1" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
     </row>
     <row r="522" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13323,10 +13332,10 @@
         <v>123</v>
       </c>
       <c r="G522" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H522" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K522" s="1" t="s">
         <v>125</v>
@@ -13340,10 +13349,10 @@
         <v>21</v>
       </c>
       <c r="G523" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H523" s="11" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="K523" s="1" t="s">
         <v>41</v>
@@ -13363,18 +13372,18 @@
         <v>17</v>
       </c>
       <c r="I524" s="6" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="J524" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L524" s="1" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
     </row>
     <row r="525" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B525" s="5" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D525" s="1" t="s">
         <v>29</v>
@@ -13409,13 +13418,13 @@
         <v>17</v>
       </c>
       <c r="I526" s="6" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="J526" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L526" s="1" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
     </row>
     <row r="527" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13426,10 +13435,10 @@
         <v>123</v>
       </c>
       <c r="G527" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H527" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K527" s="1" t="s">
         <v>125</v>
@@ -13443,10 +13452,10 @@
         <v>21</v>
       </c>
       <c r="G528" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H528" s="11" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="K528" s="1" t="s">
         <v>41</v>
@@ -13466,18 +13475,18 @@
         <v>17</v>
       </c>
       <c r="I529" s="6" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="J529" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L529" s="1" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
     </row>
     <row r="530" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B530" s="5" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="D530" s="1" t="s">
         <v>29</v>
@@ -13512,13 +13521,13 @@
         <v>17</v>
       </c>
       <c r="I531" s="6" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="J531" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L531" s="1" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
     </row>
     <row r="532" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13529,10 +13538,10 @@
         <v>123</v>
       </c>
       <c r="G532" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H532" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K532" s="1" t="s">
         <v>125</v>
@@ -13546,10 +13555,10 @@
         <v>89</v>
       </c>
       <c r="G533" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H533" s="11" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="K533" s="1" t="s">
         <v>41</v>
@@ -13563,10 +13572,10 @@
         <v>21</v>
       </c>
       <c r="G534" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H534" s="11" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
     </row>
     <row r="535" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13583,18 +13592,18 @@
         <v>17</v>
       </c>
       <c r="I535" s="6" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="J535" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L535" s="1" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="536" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B536" s="5" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D536" s="1" t="s">
         <v>29</v>
@@ -13635,7 +13644,7 @@
         <v>112</v>
       </c>
       <c r="L537" s="22" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
     </row>
     <row r="538" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13646,10 +13655,10 @@
         <v>123</v>
       </c>
       <c r="G538" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H538" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K538" s="1" t="s">
         <v>125</v>
@@ -13663,10 +13672,10 @@
         <v>89</v>
       </c>
       <c r="G539" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H539" s="11" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="K539" s="1" t="s">
         <v>41</v>
@@ -13680,10 +13689,10 @@
         <v>21</v>
       </c>
       <c r="G540" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H540" s="11" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
     </row>
     <row r="541" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13700,18 +13709,18 @@
         <v>17</v>
       </c>
       <c r="I541" s="6" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="J541" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L541" s="1" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
     </row>
     <row r="542" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B542" s="5" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="D542" s="1" t="s">
         <v>29</v>
@@ -13746,13 +13755,13 @@
         <v>17</v>
       </c>
       <c r="I543" s="6" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="J543" s="1" t="s">
         <v>177</v>
       </c>
       <c r="L543" s="1" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
     </row>
     <row r="544" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13763,10 +13772,10 @@
         <v>123</v>
       </c>
       <c r="G544" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H544" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K544" s="1" t="s">
         <v>125</v>
@@ -13780,10 +13789,10 @@
         <v>89</v>
       </c>
       <c r="G545" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H545" s="11" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="K545" s="1" t="s">
         <v>41</v>
@@ -13791,7 +13800,7 @@
     </row>
     <row r="546" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B546" s="5" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D546" s="1" t="s">
         <v>29</v>
@@ -13826,13 +13835,13 @@
         <v>17</v>
       </c>
       <c r="I547" s="6" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="J547" s="1" t="s">
         <v>177</v>
       </c>
       <c r="L547" s="1" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
     </row>
     <row r="548" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13843,10 +13852,10 @@
         <v>123</v>
       </c>
       <c r="G548" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H548" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K548" s="1" t="s">
         <v>125</v>
@@ -13860,10 +13869,10 @@
         <v>89</v>
       </c>
       <c r="G549" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H549" s="11" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="K549" s="1" t="s">
         <v>41</v>
@@ -13871,7 +13880,7 @@
     </row>
     <row r="550" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B550" s="5" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="D550" s="1" t="s">
         <v>14</v>
@@ -13906,13 +13915,13 @@
         <v>17</v>
       </c>
       <c r="I551" s="6" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="J551" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L551" s="1" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="552" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13923,10 +13932,10 @@
         <v>123</v>
       </c>
       <c r="G552" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H552" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K552" s="1" t="s">
         <v>125</v>
@@ -13940,10 +13949,10 @@
         <v>89</v>
       </c>
       <c r="G553" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H553" s="11" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="K553" s="1" t="s">
         <v>41</v>
@@ -13957,10 +13966,10 @@
         <v>21</v>
       </c>
       <c r="G554" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H554" s="11" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
     </row>
     <row r="555" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13977,18 +13986,18 @@
         <v>17</v>
       </c>
       <c r="I555" s="3" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="J555" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L555" s="1" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
     </row>
     <row r="556" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B556" s="5" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="D556" s="1" t="s">
         <v>14</v>
@@ -14023,13 +14032,13 @@
         <v>17</v>
       </c>
       <c r="I557" s="6" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="J557" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L557" s="1" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
     </row>
     <row r="558" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14040,10 +14049,10 @@
         <v>123</v>
       </c>
       <c r="G558" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H558" s="18" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="K558" s="1" t="s">
         <v>125</v>
@@ -14057,10 +14066,10 @@
         <v>89</v>
       </c>
       <c r="G559" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H559" s="11" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="K559" s="1" t="s">
         <v>41</v>
@@ -14074,10 +14083,10 @@
         <v>21</v>
       </c>
       <c r="G560" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H560" s="11" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
     </row>
     <row r="561" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14100,15 +14109,15 @@
         <v>112</v>
       </c>
       <c r="L561" s="1" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
     </row>
     <row r="562" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A562" s="4" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B562" s="5" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="D562" s="1" t="s">
         <v>29</v>
@@ -14149,7 +14158,7 @@
         <v>112</v>
       </c>
       <c r="L563" s="1" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
     </row>
     <row r="564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14166,7 +14175,7 @@
         <v>17</v>
       </c>
       <c r="I564" s="8" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="K564" s="1" t="s">
         <v>125</v>
@@ -14174,7 +14183,7 @@
     </row>
     <row r="565" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C565" s="1" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E565" s="1" t="s">
         <v>115</v>
@@ -14183,10 +14192,10 @@
         <v>279</v>
       </c>
       <c r="G565" s="1" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="H565" s="11" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="K565" s="1" t="s">
         <v>41</v>
@@ -14194,7 +14203,7 @@
     </row>
     <row r="566" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C566" s="1" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E566" s="1" t="s">
         <v>118</v>
@@ -14211,10 +14220,10 @@
     </row>
     <row r="567" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A567" s="4" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B567" s="5" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="D567" s="1" t="s">
         <v>14</v>
@@ -14249,13 +14258,13 @@
         <v>17</v>
       </c>
       <c r="I568" s="6" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="J568" s="1" t="s">
         <v>184</v>
       </c>
       <c r="L568" s="1" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
     </row>
     <row r="569" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14266,10 +14275,10 @@
         <v>89</v>
       </c>
       <c r="G569" s="1" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="H569" s="11" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="570" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14280,10 +14289,10 @@
         <v>21</v>
       </c>
       <c r="G570" s="1" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="H570" s="11" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
     </row>
     <row r="571" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14291,7 +14300,7 @@
         <v>64</v>
       </c>
       <c r="E571" s="1" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="F571" s="1" t="s">
         <v>292</v>
@@ -14309,7 +14318,7 @@
     </row>
     <row r="572" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B572" s="5" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="D572" s="1" t="s">
         <v>14</v>
@@ -14344,13 +14353,13 @@
         <v>17</v>
       </c>
       <c r="I573" s="6" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="J573" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L573" s="1" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="574" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14388,13 +14397,13 @@
         <v>17</v>
       </c>
       <c r="I575" s="6" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="J575" s="1" t="s">
         <v>56</v>
       </c>
       <c r="L575" s="1" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="576" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14405,10 +14414,10 @@
         <v>21</v>
       </c>
       <c r="G576" s="1" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="H576" s="11" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="K576" s="1" t="s">
         <v>41</v>
@@ -14416,10 +14425,10 @@
     </row>
     <row r="577" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A577" s="4" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B577" s="5" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="D577" s="1" t="s">
         <v>14</v>
@@ -14454,13 +14463,13 @@
         <v>17</v>
       </c>
       <c r="I578" s="6" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="J578" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L578" s="1" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
     </row>
     <row r="579" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14477,7 +14486,7 @@
         <v>17</v>
       </c>
       <c r="I579" s="8" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
     </row>
     <row r="580" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14494,13 +14503,13 @@
         <v>17</v>
       </c>
       <c r="I580" s="6" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="J580" s="1" t="s">
         <v>56</v>
       </c>
       <c r="L580" s="1" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
     </row>
     <row r="581" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14511,10 +14520,10 @@
         <v>279</v>
       </c>
       <c r="G581" s="1" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="H581" s="11" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="582" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14533,10 +14542,10 @@
     </row>
     <row r="583" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A583" s="4" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="B583" s="5" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="D583" s="1" t="s">
         <v>34</v>
@@ -14562,10 +14571,10 @@
         <v>141</v>
       </c>
       <c r="G584" s="1" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H584" s="11" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="J584" s="1" t="s">
         <v>143</v>
@@ -14582,10 +14591,10 @@
         <v>21</v>
       </c>
       <c r="G585" s="1" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H585" s="11" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
     </row>
     <row r="586" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14593,13 +14602,13 @@
         <v>147</v>
       </c>
       <c r="F586" s="1" t="s">
+        <v>632</v>
+      </c>
+      <c r="G586" s="1" t="s">
         <v>630</v>
       </c>
-      <c r="G586" s="1" t="s">
-        <v>628</v>
-      </c>
       <c r="H586" s="11" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="K586" s="1" t="s">
         <v>125</v>
@@ -14613,29 +14622,29 @@
         <v>89</v>
       </c>
       <c r="G587" s="1" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H587" s="11" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="588" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E588" s="1" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F588" s="1" t="s">
         <v>21</v>
       </c>
       <c r="G588" s="1" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H588" s="11" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
     </row>
     <row r="589" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B589" s="5" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D589" s="1" t="s">
         <v>29</v>
@@ -14681,10 +14690,10 @@
         <v>38</v>
       </c>
       <c r="G591" s="1" t="s">
+        <v>630</v>
+      </c>
+      <c r="H591" s="4" t="s">
         <v>628</v>
-      </c>
-      <c r="H591" s="4" t="s">
-        <v>626</v>
       </c>
       <c r="I591" s="3" t="str">
         <f aca="false">$B$583</f>
@@ -14719,10 +14728,10 @@
         <v>89</v>
       </c>
       <c r="G593" s="1" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H593" s="11" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="594" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14733,32 +14742,32 @@
         <v>21</v>
       </c>
       <c r="G594" s="1" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H594" s="11" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
     </row>
     <row r="595" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B595" s="5" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="C595" s="1" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="G595" s="23" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H595" s="15" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
     </row>
     <row r="596" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G596" s="23" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="H596" s="12" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
     </row>
     <row r="597" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14769,10 +14778,10 @@
     </row>
     <row r="601" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B601" s="5" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="G601" s="23" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="H601" s="12" t="s">
         <v>46</v>
@@ -14780,42 +14789,42 @@
     </row>
     <row r="602" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G602" s="23" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="H602" s="12" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
     </row>
     <row r="603" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G603" s="23" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="H603" s="12" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
     </row>
     <row r="604" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G604" s="23" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="H604" s="12" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
     </row>
     <row r="605" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G605" s="23" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="H605" s="12" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
     </row>
     <row r="606" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G606" s="23" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="H606" s="12" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
     </row>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
update biomarker date var
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -1770,21 +1770,21 @@
     <t xml:space="preserve">$.donors[].biomarkers[]</t>
   </si>
   <si>
+    <t xml:space="preserve">OMOP PSA Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4272032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prostate specific antigen measurement</t>
+  </si>
+  <si>
     <t xml:space="preserve">Biomarker</t>
   </si>
   <si>
     <t xml:space="preserve">test_date</t>
   </si>
   <si>
-    <t xml:space="preserve">OMOP PSA Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4272032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prostate specific antigen measurement</t>
-  </si>
-  <si>
     <t xml:space="preserve">psa_level</t>
   </si>
   <si>
@@ -1794,6 +1794,9 @@
     <t xml:space="preserve">ng/mL</t>
   </si>
   <si>
+    <t xml:space="preserve">{current_biomarker_date}</t>
+  </si>
+  <si>
     <t xml:space="preserve">OMOP CA125 Biomarker Measurement</t>
   </si>
   <si>
@@ -1917,16 +1920,13 @@
     <t xml:space="preserve">Human papillomavirus typing</t>
   </si>
   <si>
-    <t xml:space="preserve">{Biomarker.test_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biomarker – HPV strain (Code)</t>
+    <t xml:space="preserve">Biomarker - HPV strain (Code)</t>
   </si>
   <si>
     <t xml:space="preserve">hpv_strain</t>
   </si>
   <si>
-    <t xml:space="preserve">Biomarker – HPV strain (Text From Source)</t>
+    <t xml:space="preserve">Biomarker - HPV strain (Text From Source)</t>
   </si>
   <si>
     <t xml:space="preserve">$.donors[].exposures[]</t>
@@ -13150,137 +13150,136 @@
         <v>61</v>
       </c>
     </row>
-    <row r="514" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="514" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A514" s="4" t="s">
         <v>556</v>
       </c>
+      <c r="B514" s="5" t="s">
+        <v>557</v>
+      </c>
       <c r="D514" s="1" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="E514" s="1" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="F514" s="1" t="s">
-        <v>75</v>
+        <v>277</v>
       </c>
       <c r="G514" s="1" t="s">
-        <v>557</v>
-      </c>
-      <c r="H514" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H514" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K514" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="515" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E515" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F515" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G515" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H515" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I515" s="6" t="s">
         <v>558</v>
       </c>
-      <c r="I514" s="20"/>
-      <c r="K514" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="515" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A515" s="0"/>
-      <c r="B515" s="5" t="s">
+      <c r="J515" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L515" s="1" t="s">
         <v>559</v>
-      </c>
-      <c r="D515" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E515" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F515" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G515" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H515" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K515" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="516" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E516" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F516" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G516" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H516" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I516" s="6" t="s">
         <v>560</v>
       </c>
-      <c r="J516" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L516" s="1" t="s">
+      <c r="H516" s="18" t="s">
         <v>561</v>
+      </c>
+      <c r="K516" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="517" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E517" s="1" t="s">
-        <v>31</v>
+        <v>363</v>
       </c>
       <c r="F517" s="1" t="s">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="G517" s="1" t="s">
-        <v>557</v>
-      </c>
-      <c r="H517" s="18" t="s">
-        <v>558</v>
+        <v>560</v>
+      </c>
+      <c r="H517" s="11" t="s">
+        <v>562</v>
       </c>
       <c r="K517" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="518" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E518" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F518" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G518" s="1" t="s">
-        <v>557</v>
-      </c>
-      <c r="H518" s="11" t="s">
-        <v>562</v>
-      </c>
-      <c r="K518" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="519" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="H518" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I518" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="J518" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L518" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="519" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D519" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="E519" s="1" t="s">
-        <v>366</v>
+        <v>565</v>
       </c>
       <c r="F519" s="1" t="s">
-        <v>16</v>
+        <v>75</v>
       </c>
       <c r="G519" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H519" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I519" s="6" t="s">
-        <v>563</v>
-      </c>
-      <c r="J519" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L519" s="1" t="s">
-        <v>564</v>
+        <v>560</v>
+      </c>
+      <c r="H519" s="11" t="s">
+        <v>561</v>
+      </c>
+      <c r="I519" s="20"/>
+      <c r="K519" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="520" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B520" s="5" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="D520" s="1" t="s">
         <v>29</v>
@@ -13315,13 +13314,13 @@
         <v>17</v>
       </c>
       <c r="I521" s="6" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="J521" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L521" s="1" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
     </row>
     <row r="522" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13332,10 +13331,10 @@
         <v>123</v>
       </c>
       <c r="G522" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H522" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K522" s="1" t="s">
         <v>125</v>
@@ -13349,10 +13348,10 @@
         <v>21</v>
       </c>
       <c r="G523" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H523" s="11" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="K523" s="1" t="s">
         <v>41</v>
@@ -13372,18 +13371,18 @@
         <v>17</v>
       </c>
       <c r="I524" s="6" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="J524" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L524" s="1" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="525" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B525" s="5" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="D525" s="1" t="s">
         <v>29</v>
@@ -13418,13 +13417,13 @@
         <v>17</v>
       </c>
       <c r="I526" s="6" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="J526" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L526" s="1" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="527" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13435,10 +13434,10 @@
         <v>123</v>
       </c>
       <c r="G527" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H527" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K527" s="1" t="s">
         <v>125</v>
@@ -13452,10 +13451,10 @@
         <v>21</v>
       </c>
       <c r="G528" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H528" s="11" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="K528" s="1" t="s">
         <v>41</v>
@@ -13486,7 +13485,7 @@
     </row>
     <row r="530" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B530" s="5" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D530" s="1" t="s">
         <v>29</v>
@@ -13521,13 +13520,13 @@
         <v>17</v>
       </c>
       <c r="I531" s="6" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="J531" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L531" s="1" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
     </row>
     <row r="532" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13538,10 +13537,10 @@
         <v>123</v>
       </c>
       <c r="G532" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H532" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K532" s="1" t="s">
         <v>125</v>
@@ -13555,10 +13554,10 @@
         <v>89</v>
       </c>
       <c r="G533" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H533" s="11" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="K533" s="1" t="s">
         <v>41</v>
@@ -13572,10 +13571,10 @@
         <v>21</v>
       </c>
       <c r="G534" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H534" s="11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
     </row>
     <row r="535" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13592,18 +13591,18 @@
         <v>17</v>
       </c>
       <c r="I535" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="J535" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L535" s="1" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="536" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B536" s="5" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D536" s="1" t="s">
         <v>29</v>
@@ -13644,7 +13643,7 @@
         <v>112</v>
       </c>
       <c r="L537" s="22" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="538" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13655,10 +13654,10 @@
         <v>123</v>
       </c>
       <c r="G538" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H538" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K538" s="1" t="s">
         <v>125</v>
@@ -13672,10 +13671,10 @@
         <v>89</v>
       </c>
       <c r="G539" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H539" s="11" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="K539" s="1" t="s">
         <v>41</v>
@@ -13689,10 +13688,10 @@
         <v>21</v>
       </c>
       <c r="G540" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H540" s="11" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="541" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13709,18 +13708,18 @@
         <v>17</v>
       </c>
       <c r="I541" s="6" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="J541" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L541" s="1" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="542" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B542" s="5" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D542" s="1" t="s">
         <v>29</v>
@@ -13755,13 +13754,13 @@
         <v>17</v>
       </c>
       <c r="I543" s="6" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="J543" s="1" t="s">
         <v>177</v>
       </c>
       <c r="L543" s="1" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
     </row>
     <row r="544" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13772,10 +13771,10 @@
         <v>123</v>
       </c>
       <c r="G544" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H544" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K544" s="1" t="s">
         <v>125</v>
@@ -13789,10 +13788,10 @@
         <v>89</v>
       </c>
       <c r="G545" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H545" s="11" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="K545" s="1" t="s">
         <v>41</v>
@@ -13800,7 +13799,7 @@
     </row>
     <row r="546" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B546" s="5" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="D546" s="1" t="s">
         <v>29</v>
@@ -13835,13 +13834,13 @@
         <v>17</v>
       </c>
       <c r="I547" s="6" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="J547" s="1" t="s">
         <v>177</v>
       </c>
       <c r="L547" s="1" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
     </row>
     <row r="548" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13852,10 +13851,10 @@
         <v>123</v>
       </c>
       <c r="G548" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H548" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K548" s="1" t="s">
         <v>125</v>
@@ -13869,10 +13868,10 @@
         <v>89</v>
       </c>
       <c r="G549" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H549" s="11" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="K549" s="1" t="s">
         <v>41</v>
@@ -13880,7 +13879,7 @@
     </row>
     <row r="550" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B550" s="5" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="D550" s="1" t="s">
         <v>14</v>
@@ -13915,13 +13914,13 @@
         <v>17</v>
       </c>
       <c r="I551" s="6" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="J551" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L551" s="1" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="552" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13932,10 +13931,10 @@
         <v>123</v>
       </c>
       <c r="G552" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H552" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K552" s="1" t="s">
         <v>125</v>
@@ -13949,10 +13948,10 @@
         <v>89</v>
       </c>
       <c r="G553" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H553" s="11" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="K553" s="1" t="s">
         <v>41</v>
@@ -13966,10 +13965,10 @@
         <v>21</v>
       </c>
       <c r="G554" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H554" s="11" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="555" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13986,18 +13985,18 @@
         <v>17</v>
       </c>
       <c r="I555" s="3" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="J555" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L555" s="1" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
     </row>
     <row r="556" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B556" s="5" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D556" s="1" t="s">
         <v>14</v>
@@ -14032,13 +14031,13 @@
         <v>17</v>
       </c>
       <c r="I557" s="6" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="J557" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L557" s="1" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="558" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14049,10 +14048,10 @@
         <v>123</v>
       </c>
       <c r="G558" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H558" s="18" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="K558" s="1" t="s">
         <v>125</v>
@@ -14066,10 +14065,10 @@
         <v>89</v>
       </c>
       <c r="G559" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H559" s="11" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="K559" s="1" t="s">
         <v>41</v>
@@ -14083,10 +14082,10 @@
         <v>21</v>
       </c>
       <c r="G560" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H560" s="11" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="561" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14109,15 +14108,15 @@
         <v>112</v>
       </c>
       <c r="L561" s="1" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
     </row>
     <row r="562" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A562" s="4" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="B562" s="5" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D562" s="1" t="s">
         <v>29</v>
@@ -14158,7 +14157,7 @@
         <v>112</v>
       </c>
       <c r="L563" s="1" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14175,7 +14174,7 @@
         <v>17</v>
       </c>
       <c r="I564" s="8" t="s">
-        <v>606</v>
+        <v>565</v>
       </c>
       <c r="K564" s="1" t="s">
         <v>125</v>
@@ -14192,7 +14191,7 @@
         <v>279</v>
       </c>
       <c r="G565" s="1" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="H565" s="11" t="s">
         <v>608</v>

</xml_diff>

<commit_message>
rearrange biomarker date gv
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3535" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3536" uniqueCount="649">
   <si>
     <t xml:space="preserve">Source JSON Level</t>
   </si>
@@ -1770,6 +1770,15 @@
     <t xml:space="preserve">$.donors[].biomarkers[]</t>
   </si>
   <si>
+    <t xml:space="preserve">{current_biomarker_date}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biomarker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_date</t>
+  </si>
+  <si>
     <t xml:space="preserve">OMOP PSA Biomarker Measurement</t>
   </si>
   <si>
@@ -1779,12 +1788,6 @@
     <t xml:space="preserve">Prostate specific antigen measurement</t>
   </si>
   <si>
-    <t xml:space="preserve">Biomarker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_date</t>
-  </si>
-  <si>
     <t xml:space="preserve">psa_level</t>
   </si>
   <si>
@@ -1792,9 +1795,6 @@
   </si>
   <si>
     <t xml:space="preserve">ng/mL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{current_biomarker_date}</t>
   </si>
   <si>
     <t xml:space="preserve">OMOP CA125 Biomarker Measurement</t>
@@ -13150,131 +13150,135 @@
         <v>61</v>
       </c>
     </row>
-    <row r="514" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="514" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A514" s="4" t="s">
         <v>556</v>
       </c>
-      <c r="B514" s="5" t="s">
+      <c r="B514" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D514" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E514" s="1" t="s">
         <v>557</v>
       </c>
-      <c r="D514" s="1" t="s">
+      <c r="F514" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G514" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="H514" s="11" t="s">
+        <v>559</v>
+      </c>
+      <c r="I514" s="20"/>
+      <c r="K514" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="515" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A515" s="0"/>
+      <c r="B515" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="D515" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E514" s="1" t="s">
+      <c r="E515" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="F514" s="1" t="s">
+      <c r="F515" s="1" t="s">
         <v>277</v>
       </c>
-      <c r="G514" s="1" t="s">
+      <c r="G515" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="H514" s="4" t="s">
+      <c r="H515" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="K514" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="515" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E515" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="F515" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G515" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H515" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I515" s="6" t="s">
-        <v>558</v>
-      </c>
-      <c r="J515" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L515" s="1" t="s">
-        <v>559</v>
+      <c r="K515" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="516" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E516" s="1" t="s">
-        <v>31</v>
+        <v>169</v>
       </c>
       <c r="F516" s="1" t="s">
-        <v>123</v>
+        <v>16</v>
       </c>
       <c r="G516" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="H516" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="H516" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I516" s="6" t="s">
         <v>561</v>
       </c>
-      <c r="K516" s="1" t="s">
-        <v>125</v>
+      <c r="J516" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L516" s="1" t="s">
+        <v>562</v>
       </c>
     </row>
     <row r="517" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E517" s="1" t="s">
-        <v>363</v>
+        <v>31</v>
       </c>
       <c r="F517" s="1" t="s">
-        <v>21</v>
+        <v>123</v>
       </c>
       <c r="G517" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="H517" s="11" t="s">
-        <v>562</v>
+        <v>558</v>
+      </c>
+      <c r="H517" s="18" t="s">
+        <v>559</v>
       </c>
       <c r="K517" s="1" t="s">
-        <v>41</v>
+        <v>125</v>
       </c>
     </row>
     <row r="518" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E518" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="F518" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G518" s="1" t="s">
+        <v>558</v>
+      </c>
+      <c r="H518" s="11" t="s">
+        <v>563</v>
+      </c>
+      <c r="K518" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="519" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E519" s="1" t="s">
         <v>366</v>
       </c>
-      <c r="F518" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G518" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H518" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I518" s="6" t="s">
-        <v>563</v>
-      </c>
-      <c r="J518" s="1" t="s">
+      <c r="F519" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G519" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H519" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I519" s="6" t="s">
+        <v>564</v>
+      </c>
+      <c r="J519" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L518" s="1" t="s">
-        <v>564</v>
-      </c>
-    </row>
-    <row r="519" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D519" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E519" s="1" t="s">
+      <c r="L519" s="1" t="s">
         <v>565</v>
-      </c>
-      <c r="F519" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G519" s="1" t="s">
-        <v>560</v>
-      </c>
-      <c r="H519" s="11" t="s">
-        <v>561</v>
-      </c>
-      <c r="I519" s="20"/>
-      <c r="K519" s="1" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="520" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13331,10 +13335,10 @@
         <v>123</v>
       </c>
       <c r="G522" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H522" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K522" s="1" t="s">
         <v>125</v>
@@ -13348,7 +13352,7 @@
         <v>21</v>
       </c>
       <c r="G523" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H523" s="11" t="s">
         <v>569</v>
@@ -13434,10 +13438,10 @@
         <v>123</v>
       </c>
       <c r="G527" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H527" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K527" s="1" t="s">
         <v>125</v>
@@ -13451,7 +13455,7 @@
         <v>21</v>
       </c>
       <c r="G528" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H528" s="11" t="s">
         <v>575</v>
@@ -13474,13 +13478,13 @@
         <v>17</v>
       </c>
       <c r="I529" s="6" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="J529" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L529" s="1" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="530" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13537,10 +13541,10 @@
         <v>123</v>
       </c>
       <c r="G532" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H532" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K532" s="1" t="s">
         <v>125</v>
@@ -13554,7 +13558,7 @@
         <v>89</v>
       </c>
       <c r="G533" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H533" s="11" t="s">
         <v>579</v>
@@ -13571,7 +13575,7 @@
         <v>21</v>
       </c>
       <c r="G534" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H534" s="11" t="s">
         <v>580</v>
@@ -13654,10 +13658,10 @@
         <v>123</v>
       </c>
       <c r="G538" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H538" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K538" s="1" t="s">
         <v>125</v>
@@ -13671,7 +13675,7 @@
         <v>89</v>
       </c>
       <c r="G539" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H539" s="11" t="s">
         <v>585</v>
@@ -13688,7 +13692,7 @@
         <v>21</v>
       </c>
       <c r="G540" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H540" s="11" t="s">
         <v>586</v>
@@ -13771,10 +13775,10 @@
         <v>123</v>
       </c>
       <c r="G544" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H544" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K544" s="1" t="s">
         <v>125</v>
@@ -13788,7 +13792,7 @@
         <v>89</v>
       </c>
       <c r="G545" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H545" s="11" t="s">
         <v>590</v>
@@ -13851,10 +13855,10 @@
         <v>123</v>
       </c>
       <c r="G548" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H548" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K548" s="1" t="s">
         <v>125</v>
@@ -13868,7 +13872,7 @@
         <v>89</v>
       </c>
       <c r="G549" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H549" s="11" t="s">
         <v>594</v>
@@ -13931,10 +13935,10 @@
         <v>123</v>
       </c>
       <c r="G552" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H552" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K552" s="1" t="s">
         <v>125</v>
@@ -13948,7 +13952,7 @@
         <v>89</v>
       </c>
       <c r="G553" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H553" s="11" t="s">
         <v>598</v>
@@ -13965,7 +13969,7 @@
         <v>21</v>
       </c>
       <c r="G554" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H554" s="11" t="s">
         <v>598</v>
@@ -14048,10 +14052,10 @@
         <v>123</v>
       </c>
       <c r="G558" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H558" s="18" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
       <c r="K558" s="1" t="s">
         <v>125</v>
@@ -14065,7 +14069,7 @@
         <v>89</v>
       </c>
       <c r="G559" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H559" s="11" t="s">
         <v>602</v>
@@ -14082,7 +14086,7 @@
         <v>21</v>
       </c>
       <c r="G560" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H560" s="11" t="s">
         <v>602</v>
@@ -14174,7 +14178,7 @@
         <v>17</v>
       </c>
       <c r="I564" s="8" t="s">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="K564" s="1" t="s">
         <v>125</v>
@@ -14191,7 +14195,7 @@
         <v>279</v>
       </c>
       <c r="G565" s="1" t="s">
-        <v>560</v>
+        <v>558</v>
       </c>
       <c r="H565" s="11" t="s">
         <v>608</v>

</xml_diff>

<commit_message>
remove biomarker global var
</commit_message>
<xml_diff>
--- a/config/MOHCCN to OMOP CDM Map v0.5.xlsx
+++ b/config/MOHCCN to OMOP CDM Map v0.5.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3536" uniqueCount="649">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3529" uniqueCount="649">
   <si>
     <t xml:space="preserve">Source JSON Level</t>
   </si>
@@ -1770,154 +1770,154 @@
     <t xml:space="preserve">$.donors[].biomarkers[]</t>
   </si>
   <si>
+    <t xml:space="preserve">OMOP PSA Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4272032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prostate specific antigen measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biomarker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test_date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">psa_level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4120724</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ng/mL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP CA125 Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4197913</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA 125 measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ca125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4118305</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U/mL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP CEA Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4244721</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carcinoembryonic antigen measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP Estrogen Receptor Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4307360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estrogen receptor assay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">er_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">er_percent_positive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4041099</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP Progesterone Receptor Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Progesterone receptor assay measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pr_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pr_percent_positive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP HER2 IHC Status Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35918264</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HER2 IHC Summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">her2_ihc_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP HER2 ISH Status Biomarker Measurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35918706</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HER2 ISH Summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">her2_ish_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP HPV IHC Status Biomarker Observation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45763689</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human papillomavirus screening</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hpv_ihc_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">45769444</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immunohistochemistry technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP HPV PCR Status Biomarker Observation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hpv_pcr_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Polymerase chain reaction technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">$.donors[].biomarkers[].hpv_strain[]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OMOP HPV strain Biomarker Measurements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human papillomavirus typing</t>
+  </si>
+  <si>
     <t xml:space="preserve">{current_biomarker_date}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Biomarker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">test_date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP PSA Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4272032</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prostate specific antigen measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">psa_level</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4120724</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ng/mL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP CA125 Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4197913</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA 125 measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ca125</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4118305</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U/mL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP CEA Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4244721</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Carcinoembryonic antigen measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP Estrogen Receptor Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4307360</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estrogen receptor assay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">er_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">er_percent_positive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4041099</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Percent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP Progesterone Receptor Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Progesterone receptor assay measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pr_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pr_percent_positive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP HER2 IHC Status Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35918264</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HER2 IHC Summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">her2_ihc_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP HER2 ISH Status Biomarker Measurement</t>
-  </si>
-  <si>
-    <t xml:space="preserve">35918706</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HER2 ISH Summary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">her2_ish_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP HPV IHC Status Biomarker Observation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45763689</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Human papillomavirus screening</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hpv_ihc_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">45769444</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Immunohistochemistry technique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP HPV PCR Status Biomarker Observation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hpv_pcr_status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polymerase chain reaction technique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">$.donors[].biomarkers[].hpv_strain[]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OMOP HPV strain Biomarker Measurements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Human papillomavirus typing</t>
   </si>
   <si>
     <t xml:space="preserve">Biomarker - HPV strain (Code)</t>
@@ -2155,7 +2155,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2234,10 +2234,6 @@
     </xf>
     <xf numFmtId="165" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -13150,1132 +13146,1121 @@
         <v>61</v>
       </c>
     </row>
-    <row r="514" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="514" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A514" s="4" t="s">
         <v>556</v>
       </c>
-      <c r="B514" s="1" t="s">
-        <v>63</v>
+      <c r="B514" s="5" t="s">
+        <v>557</v>
       </c>
       <c r="D514" s="1" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
       <c r="E514" s="1" t="s">
-        <v>557</v>
+        <v>168</v>
       </c>
       <c r="F514" s="1" t="s">
-        <v>75</v>
+        <v>277</v>
       </c>
       <c r="G514" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H514" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K514" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="515" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E515" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F515" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G515" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H515" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I515" s="6" t="s">
         <v>558</v>
       </c>
-      <c r="H514" s="11" t="s">
+      <c r="J515" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L515" s="1" t="s">
         <v>559</v>
-      </c>
-      <c r="I514" s="20"/>
-      <c r="K514" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="515" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A515" s="0"/>
-      <c r="B515" s="5" t="s">
-        <v>560</v>
-      </c>
-      <c r="D515" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E515" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F515" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G515" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H515" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K515" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="516" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E516" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F516" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G516" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H516" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I516" s="6" t="s">
+        <v>560</v>
+      </c>
+      <c r="H516" s="18" t="s">
         <v>561</v>
       </c>
-      <c r="J516" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L516" s="1" t="s">
-        <v>562</v>
+      <c r="K516" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="517" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E517" s="1" t="s">
-        <v>31</v>
+        <v>363</v>
       </c>
       <c r="F517" s="1" t="s">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="G517" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H517" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H517" s="11" t="s">
+        <v>562</v>
       </c>
       <c r="K517" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="518" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E518" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F518" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G518" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H518" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H518" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I518" s="6" t="s">
         <v>563</v>
       </c>
-      <c r="K518" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="519" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J518" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L518" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="519" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B519" s="5" t="s">
+        <v>565</v>
+      </c>
+      <c r="D519" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E519" s="1" t="s">
-        <v>366</v>
+        <v>168</v>
       </c>
       <c r="F519" s="1" t="s">
-        <v>16</v>
+        <v>277</v>
       </c>
       <c r="G519" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H519" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I519" s="6" t="s">
-        <v>564</v>
-      </c>
-      <c r="J519" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K519" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="520" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E520" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F520" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G520" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H520" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I520" s="6" t="s">
+        <v>566</v>
+      </c>
+      <c r="J520" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L519" s="1" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="520" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B520" s="5" t="s">
-        <v>566</v>
-      </c>
-      <c r="D520" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E520" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F520" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G520" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H520" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K520" s="1" t="s">
-        <v>41</v>
+      <c r="L520" s="1" t="s">
+        <v>567</v>
       </c>
     </row>
     <row r="521" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E521" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F521" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G521" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H521" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I521" s="6" t="s">
-        <v>567</v>
-      </c>
-      <c r="J521" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L521" s="1" t="s">
-        <v>568</v>
+        <v>560</v>
+      </c>
+      <c r="H521" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K521" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="522" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E522" s="1" t="s">
-        <v>31</v>
+        <v>363</v>
       </c>
       <c r="F522" s="1" t="s">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="G522" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H522" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H522" s="11" t="s">
+        <v>568</v>
       </c>
       <c r="K522" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="523" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E523" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F523" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G523" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H523" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H523" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I523" s="6" t="s">
         <v>569</v>
       </c>
-      <c r="K523" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="524" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J523" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L523" s="1" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="524" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B524" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="D524" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E524" s="1" t="s">
-        <v>366</v>
+        <v>168</v>
       </c>
       <c r="F524" s="1" t="s">
-        <v>16</v>
+        <v>277</v>
       </c>
       <c r="G524" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H524" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I524" s="6" t="s">
-        <v>570</v>
-      </c>
-      <c r="J524" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K524" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="525" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E525" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F525" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G525" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H525" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I525" s="6" t="s">
+        <v>572</v>
+      </c>
+      <c r="J525" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L524" s="1" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="525" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B525" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="D525" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E525" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F525" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G525" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H525" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K525" s="1" t="s">
-        <v>41</v>
+      <c r="L525" s="1" t="s">
+        <v>573</v>
       </c>
     </row>
     <row r="526" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E526" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F526" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G526" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H526" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I526" s="6" t="s">
-        <v>573</v>
-      </c>
-      <c r="J526" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L526" s="1" t="s">
-        <v>574</v>
+        <v>560</v>
+      </c>
+      <c r="H526" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K526" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="527" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E527" s="1" t="s">
-        <v>31</v>
+        <v>363</v>
       </c>
       <c r="F527" s="1" t="s">
-        <v>123</v>
+        <v>21</v>
       </c>
       <c r="G527" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H527" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H527" s="11" t="s">
+        <v>574</v>
       </c>
       <c r="K527" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="528" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E528" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F528" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G528" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H528" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H528" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I528" s="6" t="s">
+        <v>563</v>
+      </c>
+      <c r="J528" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L528" s="1" t="s">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="529" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B529" s="5" t="s">
         <v>575</v>
       </c>
-      <c r="K528" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="529" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D529" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E529" s="1" t="s">
-        <v>366</v>
+        <v>168</v>
       </c>
       <c r="F529" s="1" t="s">
-        <v>16</v>
+        <v>277</v>
       </c>
       <c r="G529" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H529" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I529" s="6" t="s">
-        <v>564</v>
-      </c>
-      <c r="J529" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K529" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="530" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E530" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F530" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G530" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H530" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I530" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="J530" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L529" s="1" t="s">
-        <v>565</v>
-      </c>
-    </row>
-    <row r="530" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B530" s="5" t="s">
-        <v>576</v>
-      </c>
-      <c r="D530" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E530" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F530" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G530" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H530" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K530" s="1" t="s">
-        <v>41</v>
+      <c r="L530" s="1" t="s">
+        <v>577</v>
       </c>
     </row>
     <row r="531" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E531" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F531" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G531" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H531" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I531" s="6" t="s">
-        <v>577</v>
-      </c>
-      <c r="J531" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L531" s="1" t="s">
-        <v>578</v>
+        <v>560</v>
+      </c>
+      <c r="H531" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K531" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="532" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E532" s="1" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="F532" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="G532" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H532" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H532" s="11" t="s">
+        <v>578</v>
       </c>
       <c r="K532" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="533" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E533" s="1" t="s">
-        <v>115</v>
+        <v>363</v>
       </c>
       <c r="F533" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="G533" s="1" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="H533" s="11" t="s">
         <v>579</v>
       </c>
-      <c r="K533" s="1" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="534" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E534" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F534" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G534" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H534" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H534" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I534" s="6" t="s">
         <v>580</v>
       </c>
-    </row>
-    <row r="535" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J534" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L534" s="1" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="535" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B535" s="5" t="s">
+        <v>582</v>
+      </c>
+      <c r="D535" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E535" s="1" t="s">
-        <v>366</v>
+        <v>168</v>
       </c>
       <c r="F535" s="1" t="s">
-        <v>16</v>
+        <v>277</v>
       </c>
       <c r="G535" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H535" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I535" s="6" t="s">
-        <v>581</v>
-      </c>
-      <c r="J535" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K535" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="536" customFormat="false" ht="26.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E536" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F536" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G536" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H536" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I536" s="20" t="n">
+        <v>4030384</v>
+      </c>
+      <c r="J536" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L535" s="1" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="536" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B536" s="5" t="s">
+      <c r="L536" s="21" t="s">
         <v>583</v>
       </c>
-      <c r="D536" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E536" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F536" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G536" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H536" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K536" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="537" customFormat="false" ht="26.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="537" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E537" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F537" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G537" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H537" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I537" s="21" t="n">
-        <v>4030384</v>
-      </c>
-      <c r="J537" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L537" s="22" t="s">
-        <v>584</v>
+        <v>560</v>
+      </c>
+      <c r="H537" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K537" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="538" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E538" s="1" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="F538" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="G538" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H538" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H538" s="11" t="s">
+        <v>584</v>
       </c>
       <c r="K538" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="539" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E539" s="1" t="s">
-        <v>115</v>
+        <v>363</v>
       </c>
       <c r="F539" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="G539" s="1" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="H539" s="11" t="s">
         <v>585</v>
       </c>
-      <c r="K539" s="1" t="s">
-        <v>41</v>
-      </c>
     </row>
     <row r="540" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E540" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F540" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G540" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H540" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H540" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I540" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="J540" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L540" s="1" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="541" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B541" s="5" t="s">
         <v>586</v>
       </c>
-    </row>
-    <row r="541" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D541" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E541" s="1" t="s">
-        <v>366</v>
+        <v>168</v>
       </c>
       <c r="F541" s="1" t="s">
-        <v>16</v>
+        <v>277</v>
       </c>
       <c r="G541" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H541" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I541" s="6" t="s">
-        <v>581</v>
-      </c>
-      <c r="J541" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L541" s="1" t="s">
-        <v>582</v>
-      </c>
-    </row>
-    <row r="542" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B542" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="K541" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="542" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E542" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F542" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G542" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H542" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I542" s="6" t="s">
         <v>587</v>
       </c>
-      <c r="D542" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E542" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F542" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G542" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H542" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K542" s="1" t="s">
-        <v>41</v>
+      <c r="J542" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="L542" s="1" t="s">
+        <v>588</v>
       </c>
     </row>
     <row r="543" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E543" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F543" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G543" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H543" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I543" s="6" t="s">
-        <v>588</v>
-      </c>
-      <c r="J543" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="L543" s="1" t="s">
-        <v>589</v>
+        <v>560</v>
+      </c>
+      <c r="H543" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K543" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="544" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E544" s="1" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="F544" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="G544" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H544" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H544" s="11" t="s">
+        <v>589</v>
       </c>
       <c r="K544" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="545" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="545" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B545" s="5" t="s">
+        <v>590</v>
+      </c>
+      <c r="D545" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E545" s="1" t="s">
-        <v>115</v>
+        <v>168</v>
       </c>
       <c r="F545" s="1" t="s">
-        <v>89</v>
+        <v>277</v>
       </c>
       <c r="G545" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H545" s="11" t="s">
-        <v>590</v>
+        <v>39</v>
+      </c>
+      <c r="H545" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="K545" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="546" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B546" s="5" t="s">
+    <row r="546" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E546" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F546" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G546" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H546" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I546" s="6" t="s">
         <v>591</v>
       </c>
-      <c r="D546" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E546" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F546" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G546" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H546" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K546" s="1" t="s">
-        <v>41</v>
+      <c r="J546" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="L546" s="1" t="s">
+        <v>592</v>
       </c>
     </row>
     <row r="547" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E547" s="1" t="s">
-        <v>169</v>
+        <v>31</v>
       </c>
       <c r="F547" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G547" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H547" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I547" s="6" t="s">
-        <v>592</v>
-      </c>
-      <c r="J547" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="L547" s="1" t="s">
-        <v>593</v>
+        <v>560</v>
+      </c>
+      <c r="H547" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K547" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="548" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E548" s="1" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="F548" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="G548" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H548" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H548" s="11" t="s">
+        <v>593</v>
       </c>
       <c r="K548" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="549" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="549" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B549" s="5" t="s">
+        <v>594</v>
+      </c>
+      <c r="D549" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="E549" s="1" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="F549" s="1" t="s">
-        <v>89</v>
+        <v>277</v>
       </c>
       <c r="G549" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H549" s="11" t="s">
-        <v>594</v>
+        <v>39</v>
+      </c>
+      <c r="H549" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="K549" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="550" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B550" s="5" t="s">
+    <row r="550" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E550" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F550" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G550" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H550" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I550" s="6" t="s">
         <v>595</v>
       </c>
-      <c r="D550" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E550" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="F550" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G550" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H550" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K550" s="1" t="s">
-        <v>41</v>
+      <c r="J550" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L550" s="1" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="551" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E551" s="1" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="F551" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G551" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H551" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I551" s="6" t="s">
-        <v>596</v>
-      </c>
-      <c r="J551" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L551" s="1" t="s">
-        <v>597</v>
+        <v>560</v>
+      </c>
+      <c r="H551" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K551" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="552" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E552" s="1" t="s">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="F552" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="G552" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H552" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H552" s="11" t="s">
+        <v>597</v>
       </c>
       <c r="K552" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="553" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E553" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F553" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="G553" s="1" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="H553" s="11" t="s">
-        <v>598</v>
-      </c>
-      <c r="K553" s="1" t="s">
-        <v>41</v>
+        <v>597</v>
       </c>
     </row>
     <row r="554" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E554" s="1" t="s">
-        <v>118</v>
+        <v>216</v>
       </c>
       <c r="F554" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G554" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H554" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="H554" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I554" s="3" t="s">
         <v>598</v>
       </c>
-    </row>
-    <row r="555" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J554" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L554" s="1" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="555" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B555" s="5" t="s">
+        <v>600</v>
+      </c>
+      <c r="D555" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="E555" s="1" t="s">
-        <v>216</v>
+        <v>110</v>
       </c>
       <c r="F555" s="1" t="s">
-        <v>16</v>
+        <v>277</v>
       </c>
       <c r="G555" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H555" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I555" s="3" t="s">
-        <v>599</v>
-      </c>
-      <c r="J555" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H555" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K555" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="556" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E556" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F556" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G556" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H556" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I556" s="6" t="s">
+        <v>595</v>
+      </c>
+      <c r="J556" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="L555" s="1" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="556" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B556" s="5" t="s">
-        <v>601</v>
-      </c>
-      <c r="D556" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E556" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="F556" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G556" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H556" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K556" s="1" t="s">
-        <v>41</v>
+      <c r="L556" s="1" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="557" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E557" s="1" t="s">
-        <v>111</v>
+        <v>20</v>
       </c>
       <c r="F557" s="1" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="G557" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H557" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I557" s="6" t="s">
-        <v>596</v>
-      </c>
-      <c r="J557" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L557" s="1" t="s">
-        <v>597</v>
+        <v>560</v>
+      </c>
+      <c r="H557" s="18" t="s">
+        <v>561</v>
+      </c>
+      <c r="K557" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="558" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E558" s="1" t="s">
-        <v>20</v>
+        <v>115</v>
       </c>
       <c r="F558" s="1" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="G558" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H558" s="18" t="s">
-        <v>559</v>
+        <v>560</v>
+      </c>
+      <c r="H558" s="11" t="s">
+        <v>601</v>
       </c>
       <c r="K558" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="559" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E559" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="F559" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G559" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="H559" s="11" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="560" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E560" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="F560" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G560" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H560" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I560" s="20" t="n">
+        <v>4120014</v>
+      </c>
+      <c r="J560" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L560" s="1" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="561" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A561" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="B561" s="5" t="s">
+        <v>604</v>
+      </c>
+      <c r="D561" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E561" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F561" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="G561" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H561" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K561" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="562" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E562" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="F562" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G562" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H562" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I562" s="20" t="n">
+        <v>4194639</v>
+      </c>
+      <c r="J562" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L562" s="1" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="563" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E563" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F563" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G563" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H563" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I563" s="8" t="s">
+        <v>606</v>
+      </c>
+      <c r="K563" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C564" s="1" t="s">
+        <v>607</v>
+      </c>
+      <c r="E564" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="F559" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="G559" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H559" s="11" t="s">
-        <v>602</v>
-      </c>
-      <c r="K559" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="560" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E560" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="F560" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G560" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H560" s="11" t="s">
-        <v>602</v>
-      </c>
-    </row>
-    <row r="561" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E561" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="F561" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G561" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H561" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="I561" s="21" t="n">
-        <v>4120014</v>
-      </c>
-      <c r="J561" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L561" s="1" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="562" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A562" s="4" t="s">
-        <v>604</v>
-      </c>
-      <c r="B562" s="5" t="s">
-        <v>605</v>
-      </c>
-      <c r="D562" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E562" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="F562" s="1" t="s">
-        <v>277</v>
-      </c>
-      <c r="G562" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H562" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K562" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="563" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E563" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="F563" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="G563" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H563" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I563" s="21" t="n">
-        <v>4194639</v>
-      </c>
-      <c r="J563" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L563" s="1" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="564" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E564" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="F564" s="1" t="s">
-        <v>123</v>
+        <v>279</v>
       </c>
       <c r="G564" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H564" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I564" s="8" t="s">
-        <v>557</v>
+        <v>560</v>
+      </c>
+      <c r="H564" s="11" t="s">
+        <v>608</v>
       </c>
       <c r="K564" s="1" t="s">
-        <v>125</v>
+        <v>41</v>
       </c>
     </row>
     <row r="565" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C565" s="1" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E565" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F565" s="1" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="G565" s="1" t="s">
-        <v>558</v>
-      </c>
-      <c r="H565" s="11" t="s">
-        <v>608</v>
-      </c>
-      <c r="K565" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="566" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C566" s="1" t="s">
-        <v>609</v>
+        <v>17</v>
+      </c>
+      <c r="H565" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="566" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A566" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="B566" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="D566" s="1" t="s">
+        <v>14</v>
       </c>
       <c r="E566" s="1" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="F566" s="1" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="G566" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H566" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="567" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A567" s="4" t="s">
-        <v>610</v>
-      </c>
-      <c r="B567" s="5" t="s">
-        <v>611</v>
-      </c>
-      <c r="D567" s="1" t="s">
-        <v>14</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="K566" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="567" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E567" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F567" s="1" t="s">
-        <v>277</v>
+        <v>16</v>
       </c>
       <c r="G567" s="1" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="H567" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K567" s="1" t="s">
-        <v>41</v>
+        <v>17</v>
+      </c>
+      <c r="I567" s="6" t="s">
+        <v>612</v>
+      </c>
+      <c r="J567" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="L567" s="1" t="s">
+        <v>613</v>
       </c>
     </row>
     <row r="568" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E568" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F568" s="1" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="G568" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H568" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I568" s="6" t="s">
-        <v>612</v>
-      </c>
-      <c r="J568" s="1" t="s">
-        <v>184</v>
-      </c>
-      <c r="L568" s="1" t="s">
-        <v>613</v>
+        <v>614</v>
+      </c>
+      <c r="H568" s="11" t="s">
+        <v>615</v>
       </c>
     </row>
     <row r="569" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E569" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F569" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="G569" s="1" t="s">
         <v>614</v>
@@ -14285,28 +14270,38 @@
       </c>
     </row>
     <row r="570" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D570" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="E570" s="1" t="s">
-        <v>118</v>
+        <v>616</v>
       </c>
       <c r="F570" s="1" t="s">
-        <v>21</v>
+        <v>292</v>
       </c>
       <c r="G570" s="1" t="s">
-        <v>614</v>
-      </c>
-      <c r="H570" s="11" t="s">
-        <v>615</v>
-      </c>
-    </row>
-    <row r="571" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>39</v>
+      </c>
+      <c r="H570" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I570" s="3" t="str">
+        <f aca="false">$B$566</f>
+        <v>OMOP Tobacco Smoking Status Observation</v>
+      </c>
+    </row>
+    <row r="571" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B571" s="5" t="s">
+        <v>617</v>
+      </c>
       <c r="D571" s="1" t="s">
-        <v>64</v>
+        <v>14</v>
       </c>
       <c r="E571" s="1" t="s">
-        <v>616</v>
+        <v>110</v>
       </c>
       <c r="F571" s="1" t="s">
-        <v>292</v>
+        <v>277</v>
       </c>
       <c r="G571" s="1" t="s">
         <v>39</v>
@@ -14314,264 +14309,260 @@
       <c r="H571" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="I571" s="3" t="str">
-        <f aca="false">$B$567</f>
-        <v>OMOP Tobacco Smoking Status Observation</v>
-      </c>
-    </row>
-    <row r="572" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B572" s="5" t="s">
-        <v>617</v>
-      </c>
-      <c r="D572" s="1" t="s">
-        <v>14</v>
-      </c>
+      <c r="K571" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="572" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E572" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F572" s="1" t="s">
-        <v>277</v>
+        <v>16</v>
       </c>
       <c r="G572" s="1" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="H572" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K572" s="1" t="s">
-        <v>41</v>
+        <v>17</v>
+      </c>
+      <c r="I572" s="6" t="s">
+        <v>618</v>
+      </c>
+      <c r="J572" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L572" s="1" t="s">
+        <v>619</v>
       </c>
     </row>
     <row r="573" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E573" s="1" t="s">
-        <v>111</v>
+        <v>189</v>
       </c>
       <c r="F573" s="1" t="s">
-        <v>16</v>
+        <v>292</v>
       </c>
       <c r="G573" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H573" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I573" s="6" t="s">
-        <v>618</v>
-      </c>
-      <c r="J573" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L573" s="1" t="s">
-        <v>619</v>
+        <v>40</v>
+      </c>
+      <c r="I573" s="3" t="str">
+        <f aca="false">$B$566</f>
+        <v>OMOP Tobacco Smoking Status Observation</v>
+      </c>
+      <c r="K573" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="574" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E574" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F574" s="1" t="s">
-        <v>292</v>
+        <v>16</v>
       </c>
       <c r="G574" s="1" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="H574" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="I574" s="3" t="str">
-        <f aca="false">$B$567</f>
-        <v>OMOP Tobacco Smoking Status Observation</v>
-      </c>
-      <c r="K574" s="1" t="s">
-        <v>41</v>
+        <v>17</v>
+      </c>
+      <c r="I574" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="J574" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L574" s="1" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="575" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E575" s="1" t="s">
-        <v>190</v>
+        <v>363</v>
       </c>
       <c r="F575" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="G575" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H575" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I575" s="6" t="s">
-        <v>620</v>
-      </c>
-      <c r="J575" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="L575" s="1" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="576" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>614</v>
+      </c>
+      <c r="H575" s="11" t="s">
+        <v>622</v>
+      </c>
+      <c r="K575" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="576" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A576" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="B576" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="D576" s="1" t="s">
+        <v>14</v>
+      </c>
       <c r="E576" s="1" t="s">
-        <v>363</v>
+        <v>110</v>
       </c>
       <c r="F576" s="1" t="s">
-        <v>21</v>
+        <v>277</v>
       </c>
       <c r="G576" s="1" t="s">
-        <v>614</v>
-      </c>
-      <c r="H576" s="11" t="s">
-        <v>622</v>
+        <v>39</v>
+      </c>
+      <c r="H576" s="4" t="s">
+        <v>40</v>
       </c>
       <c r="K576" s="1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="577" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A577" s="4" t="s">
-        <v>623</v>
-      </c>
-      <c r="B577" s="5" t="s">
-        <v>624</v>
-      </c>
-      <c r="D577" s="1" t="s">
-        <v>14</v>
-      </c>
+    <row r="577" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E577" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F577" s="1" t="s">
-        <v>277</v>
+        <v>16</v>
       </c>
       <c r="G577" s="1" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="H577" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="K577" s="1" t="s">
-        <v>41</v>
+        <v>17</v>
+      </c>
+      <c r="I577" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="J577" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="L577" s="1" t="s">
+        <v>626</v>
       </c>
     </row>
     <row r="578" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E578" s="1" t="s">
-        <v>111</v>
+        <v>189</v>
       </c>
       <c r="F578" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="G578" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H578" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I578" s="6" t="s">
-        <v>625</v>
-      </c>
-      <c r="J578" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L578" s="1" t="s">
-        <v>626</v>
+      <c r="H578" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I578" s="8" t="s">
+        <v>616</v>
       </c>
     </row>
     <row r="579" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E579" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F579" s="1" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G579" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H579" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I579" s="8" t="s">
-        <v>616</v>
+      <c r="H579" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="I579" s="6" t="s">
+        <v>620</v>
+      </c>
+      <c r="J579" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="L579" s="1" t="s">
+        <v>621</v>
       </c>
     </row>
     <row r="580" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E580" s="1" t="s">
-        <v>190</v>
+        <v>115</v>
       </c>
       <c r="F580" s="1" t="s">
-        <v>16</v>
+        <v>279</v>
       </c>
       <c r="G580" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H580" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I580" s="6" t="s">
-        <v>620</v>
-      </c>
-      <c r="J580" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="L580" s="1" t="s">
-        <v>621</v>
+        <v>614</v>
+      </c>
+      <c r="H580" s="11" t="s">
+        <v>627</v>
       </c>
     </row>
     <row r="581" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E581" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F581" s="1" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="G581" s="1" t="s">
-        <v>614</v>
-      </c>
-      <c r="H581" s="11" t="s">
-        <v>627</v>
+        <v>17</v>
+      </c>
+      <c r="H581" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="582" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A582" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="B582" s="5" t="s">
+        <v>629</v>
+      </c>
+      <c r="D582" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="E582" s="1" t="s">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="F582" s="1" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="G582" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H582" s="4" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
     </row>
     <row r="583" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A583" s="4" t="s">
-        <v>628</v>
-      </c>
-      <c r="B583" s="5" t="s">
-        <v>629</v>
-      </c>
-      <c r="D583" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="E583" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F583" s="1" t="s">
-        <v>277</v>
+        <v>141</v>
       </c>
       <c r="G583" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="H583" s="4" t="s">
-        <v>40</v>
+        <v>630</v>
+      </c>
+      <c r="H583" s="11" t="s">
+        <v>631</v>
+      </c>
+      <c r="J583" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="K583" s="1" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="584" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E584" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="F584" s="1" t="s">
-        <v>141</v>
+        <v>21</v>
       </c>
       <c r="G584" s="1" t="s">
         <v>630</v>
@@ -14579,50 +14570,44 @@
       <c r="H584" s="11" t="s">
         <v>631</v>
       </c>
-      <c r="J584" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="K584" s="1" t="s">
-        <v>92</v>
-      </c>
     </row>
     <row r="585" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E585" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F585" s="1" t="s">
-        <v>21</v>
+        <v>632</v>
       </c>
       <c r="G585" s="1" t="s">
         <v>630</v>
       </c>
       <c r="H585" s="11" t="s">
-        <v>631</v>
+        <v>633</v>
+      </c>
+      <c r="K585" s="1" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="586" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E586" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F586" s="1" t="s">
-        <v>632</v>
+        <v>89</v>
       </c>
       <c r="G586" s="1" t="s">
         <v>630</v>
       </c>
       <c r="H586" s="11" t="s">
-        <v>633</v>
-      </c>
-      <c r="K586" s="1" t="s">
-        <v>125</v>
+        <v>634</v>
       </c>
     </row>
     <row r="587" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E587" s="1" t="s">
-        <v>149</v>
+        <v>635</v>
       </c>
       <c r="F587" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="G587" s="1" t="s">
         <v>630</v>
@@ -14631,104 +14616,104 @@
         <v>634</v>
       </c>
     </row>
-    <row r="588" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="588" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B588" s="5" t="s">
+        <v>636</v>
+      </c>
+      <c r="D588" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E588" s="1" t="s">
-        <v>635</v>
+        <v>168</v>
       </c>
       <c r="F588" s="1" t="s">
-        <v>21</v>
+        <v>277</v>
       </c>
       <c r="G588" s="1" t="s">
-        <v>630</v>
-      </c>
-      <c r="H588" s="11" t="s">
-        <v>634</v>
-      </c>
-    </row>
-    <row r="589" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B589" s="5" t="s">
-        <v>636</v>
-      </c>
-      <c r="D589" s="1" t="s">
-        <v>29</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="H588" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="589" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E589" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F589" s="1" t="s">
-        <v>277</v>
+        <v>16</v>
       </c>
       <c r="G589" s="1" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="H589" s="4" t="s">
-        <v>40</v>
+        <v>17</v>
+      </c>
+      <c r="I589" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="J589" s="1" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="590" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E590" s="1" t="s">
-        <v>169</v>
+        <v>43</v>
       </c>
       <c r="F590" s="1" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="G590" s="1" t="s">
-        <v>17</v>
+        <v>630</v>
       </c>
       <c r="H590" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I590" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="J590" s="1" t="s">
-        <v>177</v>
+        <v>628</v>
+      </c>
+      <c r="I590" s="3" t="str">
+        <f aca="false">$B$582</f>
+        <v>OMOP Comorbidity Condition</v>
       </c>
     </row>
     <row r="591" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E591" s="1" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="F591" s="1" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="G591" s="1" t="s">
-        <v>630</v>
+        <v>17</v>
       </c>
       <c r="H591" s="4" t="s">
-        <v>628</v>
-      </c>
-      <c r="I591" s="3" t="str">
-        <f aca="false">$B$583</f>
-        <v>OMOP Comorbidity Condition</v>
+        <v>17</v>
+      </c>
+      <c r="I591" s="3" t="n">
+        <v>1147127</v>
+      </c>
+      <c r="J591" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="592" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E592" s="1" t="s">
-        <v>53</v>
+        <v>115</v>
       </c>
       <c r="F592" s="1" t="s">
-        <v>16</v>
+        <v>89</v>
       </c>
       <c r="G592" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="H592" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I592" s="3" t="n">
-        <v>1147127</v>
-      </c>
-      <c r="J592" s="1" t="s">
-        <v>56</v>
+        <v>630</v>
+      </c>
+      <c r="H592" s="11" t="s">
+        <v>637</v>
       </c>
     </row>
     <row r="593" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E593" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F593" s="1" t="s">
-        <v>89</v>
+        <v>21</v>
       </c>
       <c r="G593" s="1" t="s">
         <v>630</v>
@@ -14737,99 +14722,86 @@
         <v>637</v>
       </c>
     </row>
-    <row r="594" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E594" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="F594" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G594" s="1" t="s">
+    <row r="594" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B594" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="C594" s="1" t="s">
+        <v>639</v>
+      </c>
+      <c r="G594" s="22" t="s">
         <v>630</v>
       </c>
-      <c r="H594" s="11" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="595" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B595" s="5" t="s">
-        <v>638</v>
-      </c>
-      <c r="C595" s="1" t="s">
-        <v>639</v>
-      </c>
-      <c r="G595" s="23" t="s">
+      <c r="H594" s="15" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="595" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G595" s="22" t="s">
         <v>630</v>
       </c>
-      <c r="H595" s="15" t="s">
-        <v>640</v>
+      <c r="H595" s="12" t="s">
+        <v>641</v>
       </c>
     </row>
     <row r="596" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G596" s="23" t="s">
-        <v>630</v>
-      </c>
-      <c r="H596" s="12" t="s">
-        <v>641</v>
-      </c>
+      <c r="H596" s="11"/>
     </row>
     <row r="597" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H597" s="11"/>
     </row>
-    <row r="598" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H598" s="11"/>
-    </row>
-    <row r="601" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B601" s="5" t="s">
+    <row r="600" customFormat="false" ht="24.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B600" s="5" t="s">
         <v>642</v>
       </c>
-      <c r="G601" s="23" t="s">
+      <c r="G600" s="22" t="s">
         <v>643</v>
       </c>
+      <c r="H600" s="12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="601" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G601" s="22" t="s">
+        <v>643</v>
+      </c>
       <c r="H601" s="12" t="s">
-        <v>46</v>
+        <v>644</v>
       </c>
     </row>
     <row r="602" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G602" s="23" t="s">
+      <c r="G602" s="22" t="s">
         <v>643</v>
       </c>
       <c r="H602" s="12" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="603" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G603" s="23" t="s">
+      <c r="G603" s="22" t="s">
         <v>643</v>
       </c>
       <c r="H603" s="12" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
     </row>
     <row r="604" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G604" s="23" t="s">
+      <c r="G604" s="22" t="s">
         <v>643</v>
       </c>
       <c r="H604" s="12" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
     </row>
     <row r="605" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G605" s="23" t="s">
+      <c r="G605" s="22" t="s">
         <v>643</v>
       </c>
       <c r="H605" s="12" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="606" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G606" s="23" t="s">
-        <v>643</v>
-      </c>
-      <c r="H606" s="12" t="s">
         <v>648</v>
       </c>
     </row>
+    <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>